<commit_message>
data: 0 step updates + 3 account events (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team X" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Team X" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Log" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -200,7 +200,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -270,6 +270,7 @@
     <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -595,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-20 18:45 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-20 19:59 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1372,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1427,6 +1428,78 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n"/>
+      <c r="G4" s="27" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: 0 step updates + 6 account events (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-20 19:59 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-20 21:00 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1431,7 +1431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1455,7 +1455,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1479,7 +1479,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1494,11 +1494,155 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F4" s="27" t="n"/>
       <c r="G4" s="27" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:27:02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 0 step updates + 5 account events (helbert)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-20 21:00 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-20 21:25 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1431,22 +1431,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F2" s="27" t="n"/>
@@ -1455,22 +1455,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1479,22 +1479,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F4" s="27" t="n"/>
@@ -1503,22 +1503,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F5" s="27" t="n"/>
@@ -1527,22 +1527,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F6" s="27" t="n"/>
@@ -1551,7 +1551,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1575,7 +1575,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -1623,7 +1623,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1638,11 +1638,131 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
       <c r="G10" s="27" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n"/>
+      <c r="G13" s="27" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 0 step updates + 1 account event (helbert)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-20 21:25 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-20 22:14 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1373,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1431,7 +1431,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F2" s="27" t="n"/>
@@ -1455,7 +1455,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1470,7 +1470,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1479,7 +1479,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1494,7 +1494,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F4" s="27" t="n"/>
@@ -1503,7 +1503,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F5" s="27" t="n"/>
@@ -1527,7 +1527,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F6" s="27" t="n"/>
@@ -1551,22 +1551,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F7" s="27" t="n"/>
@@ -1575,7 +1575,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1599,7 +1599,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -1623,7 +1623,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1638,7 +1638,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1647,7 +1647,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F11" s="27" t="n"/>
@@ -1671,7 +1671,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F12" s="27" t="n"/>
@@ -1695,7 +1695,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1719,7 +1719,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F14" s="27" t="n"/>
@@ -1743,7 +1743,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1758,11 +1758,35 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F15" s="27" t="n"/>
       <c r="G15" s="27" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update + 1 account event (rogelio)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-20 22:14 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-21 05:15 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -852,7 +852,9 @@
         <f>SUM(E3:AE3)</f>
         <v/>
       </c>
-      <c r="E3" s="22" t="n"/>
+      <c r="E3" s="22" t="n">
+        <v>6310</v>
+      </c>
       <c r="F3" s="22" t="n"/>
       <c r="G3" s="22" t="n"/>
       <c r="H3" s="22" t="n"/>
@@ -1373,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1431,46 +1433,58 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G2" s="27" t="n"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1479,7 +1493,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1503,7 +1517,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1527,7 +1541,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1542,7 +1556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F6" s="27" t="n"/>
@@ -1551,7 +1565,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1566,7 +1580,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F7" s="27" t="n"/>
@@ -1575,22 +1589,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F8" s="27" t="n"/>
@@ -1599,22 +1613,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -1623,7 +1637,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1638,7 +1652,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1647,7 +1661,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1671,7 +1685,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1695,7 +1709,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1719,7 +1733,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1734,7 +1748,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F14" s="27" t="n"/>
@@ -1743,7 +1757,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1758,7 +1772,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F15" s="27" t="n"/>
@@ -1767,7 +1781,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1782,11 +1796,59 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F16" s="27" t="n"/>
       <c r="G16" s="27" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates + 3 account events (luis, eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-21 05:15 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-21 12:04 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -986,8 +986,12 @@
         <f>SUM(E6:AE6)</f>
         <v/>
       </c>
-      <c r="E6" s="22" t="n"/>
-      <c r="F6" s="22" t="n"/>
+      <c r="E6" s="22" t="n">
+        <v>9060</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>100</v>
+      </c>
       <c r="G6" s="22" t="n"/>
       <c r="H6" s="22" t="n"/>
       <c r="I6" s="22" t="n"/>
@@ -1375,7 +1379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1433,17 +1437,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1453,11 +1457,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>6310</v>
+        <v>100</v>
       </c>
       <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
@@ -1469,46 +1473,58 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G3" s="27" t="n"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F4" s="27" t="n"/>
@@ -1517,22 +1533,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F5" s="27" t="n"/>
@@ -1541,17 +1557,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1565,46 +1581,58 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G7" s="27" t="n"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F8" s="27" t="n"/>
@@ -1613,7 +1641,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1637,22 +1665,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1661,22 +1689,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F11" s="27" t="n"/>
@@ -1685,22 +1713,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F12" s="27" t="n"/>
@@ -1709,22 +1737,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F13" s="27" t="n"/>
@@ -1733,22 +1761,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F14" s="27" t="n"/>
@@ -1757,7 +1785,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1781,7 +1809,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1805,7 +1833,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1820,7 +1848,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F17" s="27" t="n"/>
@@ -1829,7 +1857,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1844,11 +1872,131 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
       <c r="G18" s="27" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n"/>
+      <c r="G20" s="27" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
+      <c r="G21" s="27" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n"/>
+      <c r="G22" s="27" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
+      <c r="G23" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update + 4 account events (gonza, danielle)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-21 12:04 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-21 13:40 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -898,7 +898,9 @@
         <f>SUM(E4:AE4)</f>
         <v/>
       </c>
-      <c r="E4" s="22" t="n"/>
+      <c r="E4" s="22" t="n">
+        <v>10383</v>
+      </c>
       <c r="F4" s="22" t="n"/>
       <c r="G4" s="22" t="n"/>
       <c r="H4" s="22" t="n"/>
@@ -1379,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1437,118 +1439,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
       <c r="G2" s="27" t="n"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
       <c r="G3" s="27" t="n"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G4" s="27" t="n"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F5" s="27" t="n"/>
@@ -1557,17 +1547,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1581,17 +1571,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1601,11 +1591,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>6310</v>
+        <v>100</v>
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
@@ -1617,46 +1607,58 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G8" s="27" t="n"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -1665,22 +1667,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1689,17 +1691,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1713,46 +1715,58 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G12" s="27" t="n"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F13" s="27" t="n"/>
@@ -1761,7 +1775,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1785,22 +1799,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F15" s="27" t="n"/>
@@ -1809,22 +1823,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F16" s="27" t="n"/>
@@ -1833,22 +1847,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F17" s="27" t="n"/>
@@ -1857,22 +1871,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
@@ -1881,22 +1895,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F19" s="27" t="n"/>
@@ -1905,7 +1919,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1929,7 +1943,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1953,7 +1967,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1968,7 +1982,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F22" s="27" t="n"/>
@@ -1977,7 +1991,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1992,11 +2006,131 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n"/>
+      <c r="G24" s="27" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
+      <c r="G25" s="27" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="27" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n"/>
+      <c r="G27" s="27" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-21 13:40 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-21 15:12 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -992,7 +992,7 @@
         <v>9060</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>100</v>
+        <v>1985</v>
       </c>
       <c r="G6" s="22" t="n"/>
       <c r="H6" s="22" t="n"/>
@@ -1381,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1439,31 +1439,45 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n"/>
-      <c r="G2" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G2" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1478,7 +1492,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1487,43 +1501,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n"/>
       <c r="G4" s="27" t="n"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1538,16 +1540,28 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G5" s="27" t="n"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1562,7 +1576,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F6" s="27" t="n"/>
@@ -1571,43 +1585,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n"/>
       <c r="G7" s="27" t="n"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1627,11 +1629,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
@@ -1643,31 +1645,43 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G9" s="27" t="n"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1682,7 +1696,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1691,7 +1705,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1706,7 +1720,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F11" s="27" t="n"/>
@@ -1715,43 +1729,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n"/>
       <c r="G12" s="27" t="n"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1766,26 +1768,38 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1799,7 +1813,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1814,7 +1828,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F15" s="27" t="n"/>
@@ -1823,7 +1837,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1838,7 +1852,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F16" s="27" t="n"/>
@@ -1847,7 +1861,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1862,7 +1876,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F17" s="27" t="n"/>
@@ -1871,7 +1885,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1886,7 +1900,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
@@ -1895,7 +1909,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1910,7 +1924,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F19" s="27" t="n"/>
@@ -1919,22 +1933,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F20" s="27" t="n"/>
@@ -1943,7 +1957,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1967,7 +1981,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1982,7 +1996,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F22" s="27" t="n"/>
@@ -1991,7 +2005,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2006,7 +2020,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F23" s="27" t="n"/>
@@ -2015,7 +2029,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2030,7 +2044,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2039,7 +2053,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2054,7 +2068,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F25" s="27" t="n"/>
@@ -2063,7 +2077,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2087,7 +2101,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2102,7 +2116,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F27" s="27" t="n"/>
@@ -2111,7 +2125,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2126,11 +2140,35 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
       <c r="G28" s="27" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n"/>
+      <c r="G29" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 3 step updates + 5 account events (armando, minerva, luis)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-21 22:25 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-22 00:45 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1081,7 +1081,9 @@
         <v/>
       </c>
       <c r="E8" s="22" t="n"/>
-      <c r="F8" s="22" t="n"/>
+      <c r="F8" s="22" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" s="22" t="n"/>
       <c r="H8" s="22" t="n"/>
       <c r="I8" s="22" t="n"/>
@@ -1168,7 +1170,9 @@
         <f>SUM(E10:AE10)</f>
         <v/>
       </c>
-      <c r="E10" s="22" t="n"/>
+      <c r="E10" s="22" t="n">
+        <v>5345</v>
+      </c>
       <c r="F10" s="22" t="n"/>
       <c r="G10" s="22" t="n"/>
       <c r="H10" s="22" t="n"/>
@@ -1212,7 +1216,9 @@
         <f>SUM(E11:AE11)</f>
         <v/>
       </c>
-      <c r="E11" s="22" t="n"/>
+      <c r="E11" s="22" t="n">
+        <v>12641</v>
+      </c>
       <c r="F11" s="22" t="n"/>
       <c r="G11" s="22" t="n"/>
       <c r="H11" s="22" t="n"/>
@@ -1381,7 +1387,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1439,17 +1445,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1463,36 +1469,34 @@
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1501,22 +1505,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F4" s="27" t="n"/>
@@ -1525,17 +1529,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1549,7 +1553,7 @@
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>10383</v>
+        <v>12641</v>
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
@@ -1561,22 +1565,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F6" s="27" t="n"/>
@@ -1585,137 +1589,139 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G7" s="27" t="n"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n"/>
       <c r="G8" s="27" t="n"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
       <c r="G9" s="27" t="n"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n"/>
-      <c r="G10" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1729,17 +1735,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1753,17 +1759,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1777,7 +1783,7 @@
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>6310</v>
+        <v>10383</v>
       </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" t="inlineStr">
@@ -1789,22 +1795,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F14" s="27" t="n"/>
@@ -1813,17 +1819,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1837,70 +1843,94 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G16" s="27" t="n"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G17" s="27" t="n"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
@@ -1909,22 +1939,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F19" s="27" t="n"/>
@@ -1933,17 +1963,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1957,46 +1987,58 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G21" s="27" t="n"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F22" s="27" t="n"/>
@@ -2005,22 +2047,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F23" s="27" t="n"/>
@@ -2029,22 +2071,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2053,22 +2095,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F25" s="27" t="n"/>
@@ -2077,22 +2119,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F26" s="27" t="n"/>
@@ -2101,22 +2143,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F27" s="27" t="n"/>
@@ -2125,22 +2167,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2149,7 +2191,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2164,11 +2206,203 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F29" s="27" t="n"/>
       <c r="G29" s="27" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:41:34</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n"/>
+      <c r="G30" s="27" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:41:28</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
+      <c r="G31" s="27" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:27:02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="n"/>
+      <c r="G32" s="27" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
+      <c r="G34" s="27" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
+      <c r="G35" s="27" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update + 1 story (eron, armando)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-22 03:44 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-22 05:24 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1173,7 +1173,9 @@
       <c r="E10" s="22" t="n">
         <v>5345</v>
       </c>
-      <c r="F10" s="22" t="n"/>
+      <c r="F10" s="22" t="n">
+        <v>4842</v>
+      </c>
       <c r="G10" s="22" t="n"/>
       <c r="H10" s="22" t="n"/>
       <c r="I10" s="22" t="n"/>
@@ -1387,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1445,17 +1447,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1469,34 +1471,34 @@
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1505,67 +1507,67 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G4" s="27" t="n"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n"/>
       <c r="G5" s="27" t="n"/>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1580,7 +1582,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F6" s="27" t="n"/>
@@ -1589,17 +1591,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1613,7 +1615,7 @@
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>5345</v>
+        <v>12641</v>
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
@@ -1625,22 +1627,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F8" s="27" t="n"/>
@@ -1649,7 +1651,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1664,69 +1666,67 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G9" s="27" t="n"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G10" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F11" s="27" t="n"/>
@@ -1735,82 +1735,84 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n"/>
-      <c r="G12" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G12" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n"/>
       <c r="G13" s="27" t="n"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F14" s="27" t="n"/>
@@ -1819,7 +1821,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1834,136 +1836,148 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G15" s="27" t="n"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
       <c r="G16" s="27" t="n"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
       <c r="G17" s="27" t="n"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G18" s="27" t="n"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G19" s="27" t="n"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1978,7 +1992,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F20" s="27" t="n"/>
@@ -1987,53 +2001,41 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
       <c r="G21" s="27" t="n"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2047,46 +2049,58 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G23" s="27" t="n"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2095,7 +2109,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2119,7 +2133,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2143,7 +2157,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2158,7 +2172,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F27" s="27" t="n"/>
@@ -2167,7 +2181,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2182,7 +2196,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2191,22 +2205,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F29" s="27" t="n"/>
@@ -2215,22 +2229,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F30" s="27" t="n"/>
@@ -2239,7 +2253,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2254,7 +2268,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F31" s="27" t="n"/>
@@ -2263,7 +2277,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2287,7 +2301,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2311,7 +2325,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2335,7 +2349,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2350,7 +2364,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F35" s="27" t="n"/>
@@ -2359,7 +2373,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2374,7 +2388,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F36" s="27" t="n"/>
@@ -2383,7 +2397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2398,11 +2412,59 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F37" s="27" t="n"/>
       <c r="G37" s="27" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n"/>
+      <c r="G38" s="27" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="n"/>
+      <c r="G39" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 story + 1 account event (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-22 05:24 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-22 10:29 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1447,43 +1447,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
       <c r="G2" s="27" t="n"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1498,7 +1486,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1507,17 +1495,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1531,34 +1519,34 @@
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F5" s="27" t="n"/>
@@ -1567,67 +1555,67 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" s="27" t="n"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n"/>
       <c r="G7" s="27" t="n"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1642,7 +1630,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F8" s="27" t="n"/>
@@ -1651,17 +1639,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1675,7 +1663,7 @@
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>5345</v>
+        <v>12641</v>
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
@@ -1687,22 +1675,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1711,7 +1699,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1726,69 +1714,67 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G11" s="27" t="n"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F13" s="27" t="n"/>
@@ -1797,82 +1783,84 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n"/>
       <c r="G15" s="27" t="n"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F16" s="27" t="n"/>
@@ -1881,7 +1869,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1896,136 +1884,148 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G17" s="27" t="n"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
       <c r="G18" s="27" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n"/>
       <c r="G19" s="27" t="n"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G20" s="27" t="n"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G21" s="27" t="n"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F22" s="27" t="n"/>
@@ -2049,53 +2049,41 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2109,46 +2097,58 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G25" s="27" t="n"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F26" s="27" t="n"/>
@@ -2157,7 +2157,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2181,7 +2181,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2205,7 +2205,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F29" s="27" t="n"/>
@@ -2229,7 +2229,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2244,7 +2244,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F30" s="27" t="n"/>
@@ -2253,22 +2253,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F31" s="27" t="n"/>
@@ -2277,22 +2277,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2301,7 +2301,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2316,7 +2316,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F33" s="27" t="n"/>
@@ -2325,7 +2325,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2349,7 +2349,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2373,7 +2373,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2397,7 +2397,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F37" s="27" t="n"/>
@@ -2421,7 +2421,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F38" s="27" t="n"/>
@@ -2445,7 +2445,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2460,11 +2460,59 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
       <c r="G39" s="27" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="n"/>
+      <c r="G41" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-22 10:29 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-22 10:52 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -992,9 +992,11 @@
         <v>9060</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G6" s="22" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G6" s="22" t="n">
+        <v>1100</v>
+      </c>
       <c r="H6" s="22" t="n"/>
       <c r="I6" s="22" t="n"/>
       <c r="J6" s="22" t="n"/>
@@ -1389,7 +1391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1447,7 +1449,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1462,16 +1464,28 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G2" s="27" t="n"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1486,52 +1500,54 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n"/>
-      <c r="G3" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n"/>
       <c r="G4" s="27" t="n"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1546,7 +1562,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F5" s="27" t="n"/>
@@ -1555,17 +1571,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1579,34 +1595,34 @@
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F7" s="27" t="n"/>
@@ -1615,67 +1631,67 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G8" s="27" t="n"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
       <c r="G9" s="27" t="n"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1690,7 +1706,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1699,17 +1715,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1723,7 +1739,7 @@
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>5345</v>
+        <v>12641</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
@@ -1735,22 +1751,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F12" s="27" t="n"/>
@@ -1759,7 +1775,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1774,69 +1790,67 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F15" s="27" t="n"/>
@@ -1845,82 +1859,84 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n"/>
-      <c r="G16" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G16" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
       <c r="G17" s="27" t="n"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
@@ -1929,7 +1945,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1944,136 +1960,148 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G19" s="27" t="n"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n"/>
       <c r="G20" s="27" t="n"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
       <c r="G21" s="27" t="n"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G22" s="27" t="n"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G23" s="27" t="n"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2088,7 +2116,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2097,53 +2125,41 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
       <c r="G25" s="27" t="n"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2157,46 +2173,58 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G27" s="27" t="n"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2205,7 +2233,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2229,7 +2257,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2253,7 +2281,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2268,7 +2296,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F31" s="27" t="n"/>
@@ -2277,7 +2305,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2292,7 +2320,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2301,22 +2329,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F33" s="27" t="n"/>
@@ -2325,22 +2353,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F34" s="27" t="n"/>
@@ -2349,7 +2377,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2364,7 +2392,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F35" s="27" t="n"/>
@@ -2373,7 +2401,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2397,7 +2425,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2421,7 +2449,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2445,7 +2473,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2460,7 +2488,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2469,7 +2497,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2484,7 +2512,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F40" s="27" t="n"/>
@@ -2493,7 +2521,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2508,11 +2536,59 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F41" s="27" t="n"/>
       <c r="G41" s="27" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n"/>
+      <c r="G42" s="27" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n"/>
+      <c r="G43" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 story + 2 account events (eron, gonza)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-22 10:52 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-22 15:22 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1391,7 +1391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1449,81 +1449,55 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
       <c r="G2" s="27" t="n"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G3" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1547,7 +1521,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1562,26 +1536,38 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G5" s="27" t="n"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1595,9 +1581,11 @@
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>4842</v>
-      </c>
-      <c r="G6" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>app</t>
@@ -1607,7 +1595,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1631,82 +1619,82 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n"/>
       <c r="G8" s="27" t="n"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G9" s="27" t="n"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F10" s="27" t="n"/>
@@ -1715,17 +1703,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1735,38 +1723,38 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>12641</v>
+        <v>0</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F12" s="27" t="n"/>
@@ -1775,77 +1763,77 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n"/>
       <c r="G13" s="27" t="n"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G14" s="27" t="n"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1859,17 +1847,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1879,15 +1867,13 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>5345</v>
+      </c>
+      <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>app</t>
@@ -1897,17 +1883,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1921,17 +1907,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1945,17 +1931,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1965,13 +1951,15 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>10383</v>
-      </c>
-      <c r="G19" s="27" t="n"/>
+        <v>1985</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>app</t>
@@ -1981,22 +1969,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F20" s="27" t="n"/>
@@ -2005,17 +1993,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2029,17 +2017,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2049,11 +2037,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>100</v>
+        <v>10383</v>
       </c>
       <c r="G22" s="27" t="n"/>
       <c r="H22" t="inlineStr">
@@ -2065,58 +2053,46 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2125,106 +2101,118 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G25" s="27" t="n"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G26" s="27" t="n"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n"/>
       <c r="G27" s="27" t="n"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2233,17 +2221,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2257,41 +2245,53 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G30" s="27" t="n"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2305,7 +2305,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2329,7 +2329,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F33" s="27" t="n"/>
@@ -2353,7 +2353,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2377,22 +2377,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F35" s="27" t="n"/>
@@ -2401,22 +2401,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F36" s="27" t="n"/>
@@ -2425,22 +2425,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F37" s="27" t="n"/>
@@ -2449,7 +2449,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2473,7 +2473,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2497,7 +2497,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2512,7 +2512,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F40" s="27" t="n"/>
@@ -2521,7 +2521,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2545,7 +2545,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2569,7 +2569,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2584,11 +2584,83 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F43" s="27" t="n"/>
       <c r="G43" s="27" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n"/>
+      <c r="G44" s="27" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="n"/>
+      <c r="G45" s="27" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n"/>
+      <c r="G46" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates + 2 account events (luis, minerva, gonza)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-22 15:22 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-22 19:17 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1086,7 +1086,9 @@
       <c r="F8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="22" t="n"/>
+      <c r="G8" s="22" t="n">
+        <v>0</v>
+      </c>
       <c r="H8" s="22" t="n"/>
       <c r="I8" s="22" t="n"/>
       <c r="J8" s="22" t="n"/>
@@ -1223,7 +1225,9 @@
       <c r="E11" s="22" t="n">
         <v>12641</v>
       </c>
-      <c r="F11" s="22" t="n"/>
+      <c r="F11" s="22" t="n">
+        <v>10808</v>
+      </c>
       <c r="G11" s="22" t="n"/>
       <c r="H11" s="22" t="n"/>
       <c r="I11" s="22" t="n"/>
@@ -1391,7 +1395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1449,7 +1453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1473,7 +1477,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1497,41 +1501,53 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G4" s="27" t="n"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1545,72 +1561,58 @@
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G6" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n"/>
+      <c r="G6" s="27" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F7" s="27" t="n"/>
@@ -1619,7 +1621,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1634,7 +1636,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F8" s="27" t="n"/>
@@ -1643,17 +1645,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1663,11 +1665,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>4842</v>
+        <v>1100</v>
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
@@ -1679,7 +1681,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1694,67 +1696,69 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n"/>
-      <c r="G10" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n"/>
       <c r="G11" s="27" t="n"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F12" s="27" t="n"/>
@@ -1763,137 +1767,137 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n"/>
       <c r="G14" s="27" t="n"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G15" s="27" t="n"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
       <c r="G16" s="27" t="n"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1907,108 +1911,118 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G18" s="27" t="n"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G19" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="27" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G20" s="27" t="n"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F21" s="27" t="n"/>
@@ -2017,82 +2031,84 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n"/>
       <c r="G22" s="27" t="n"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n"/>
-      <c r="G23" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G23" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2101,53 +2117,41 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
       <c r="G25" s="27" t="n"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2161,7 +2165,7 @@
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>9060</v>
+        <v>10383</v>
       </c>
       <c r="G26" s="27" t="n"/>
       <c r="H26" t="inlineStr">
@@ -2173,17 +2177,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2197,22 +2201,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2221,41 +2225,53 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G29" s="27" t="n"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2269,7 +2285,7 @@
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>6310</v>
+        <v>9060</v>
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
@@ -2281,22 +2297,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F31" s="27" t="n"/>
@@ -2305,22 +2321,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2329,22 +2345,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F33" s="27" t="n"/>
@@ -2353,46 +2369,58 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F35" s="27" t="n"/>
@@ -2401,7 +2429,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2416,7 +2444,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F36" s="27" t="n"/>
@@ -2425,7 +2453,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2440,7 +2468,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F37" s="27" t="n"/>
@@ -2449,22 +2477,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F38" s="27" t="n"/>
@@ -2473,22 +2501,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2497,22 +2525,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F40" s="27" t="n"/>
@@ -2521,22 +2549,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F41" s="27" t="n"/>
@@ -2545,7 +2573,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2560,7 +2588,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2569,7 +2597,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2593,7 +2621,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2608,7 +2636,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2617,7 +2645,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2632,7 +2660,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2641,7 +2669,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2656,11 +2684,107 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F46" s="27" t="n"/>
       <c r="G46" s="27" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F47" s="27" t="n"/>
+      <c r="G47" s="27" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n"/>
+      <c r="G48" s="27" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F49" s="27" t="n"/>
+      <c r="G49" s="27" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F50" s="27" t="n"/>
+      <c r="G50" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update (armando)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-22 19:17 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-23 05:24 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1180,7 +1180,9 @@
       <c r="F10" s="22" t="n">
         <v>4842</v>
       </c>
-      <c r="G10" s="22" t="n"/>
+      <c r="G10" s="22" t="n">
+        <v>9097</v>
+      </c>
       <c r="H10" s="22" t="n"/>
       <c r="I10" s="22" t="n"/>
       <c r="J10" s="22" t="n"/>
@@ -1395,7 +1397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H50"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1453,31 +1455,43 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G2" s="27" t="n"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1492,7 +1506,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F3" s="27" t="n"/>
@@ -1501,53 +1515,41 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n"/>
       <c r="G4" s="27" t="n"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1557,47 +1559,59 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>0</v>
+        <v>10808</v>
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G6" s="27" t="n"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1612,7 +1626,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F7" s="27" t="n"/>
@@ -1621,22 +1635,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F8" s="27" t="n"/>
@@ -1645,7 +1659,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1660,28 +1674,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
       <c r="G9" s="27" t="n"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1701,15 +1703,13 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G10" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G10" s="27" t="n"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>app</t>
@@ -1719,7 +1719,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1734,16 +1734,30 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n"/>
-      <c r="G11" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1758,7 +1772,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F12" s="27" t="n"/>
@@ -1767,103 +1781,91 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n"/>
       <c r="G13" s="27" t="n"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G14" s="27" t="n"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n"/>
       <c r="G15" s="27" t="n"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1878,31 +1880,43 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G16" s="27" t="n"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F17" s="27" t="n"/>
@@ -1911,7 +1925,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1926,28 +1940,16 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
       <c r="G18" s="27" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1962,52 +1964,52 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G19" s="27" t="n"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n"/>
       <c r="G20" s="27" t="n"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2022,16 +2024,28 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G21" s="27" t="n"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2046,7 +2060,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F22" s="27" t="n"/>
@@ -2055,69 +2069,69 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G23" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
+      <c r="G23" s="27" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n"/>
-      <c r="G24" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G24" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2132,7 +2146,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F25" s="27" t="n"/>
@@ -2141,43 +2155,31 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n"/>
       <c r="G26" s="27" t="n"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2192,16 +2194,28 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G27" s="27" t="n"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2216,7 +2230,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2225,43 +2239,31 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n"/>
       <c r="G29" s="27" t="n"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2281,11 +2283,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
@@ -2297,31 +2299,43 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G31" s="27" t="n"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2336,7 +2350,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2345,7 +2359,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2360,7 +2374,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F33" s="27" t="n"/>
@@ -2369,43 +2383,31 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
       <c r="G34" s="27" t="n"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2420,26 +2422,38 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G35" s="27" t="n"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2453,7 +2467,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2468,7 +2482,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F37" s="27" t="n"/>
@@ -2477,7 +2491,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2492,7 +2506,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F38" s="27" t="n"/>
@@ -2501,7 +2515,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2516,7 +2530,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2525,7 +2539,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2540,7 +2554,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F40" s="27" t="n"/>
@@ -2549,7 +2563,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2564,7 +2578,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F41" s="27" t="n"/>
@@ -2573,22 +2587,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2597,7 +2611,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2621,7 +2635,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2636,7 +2650,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2645,7 +2659,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2660,7 +2674,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2669,7 +2683,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2684,7 +2698,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F46" s="27" t="n"/>
@@ -2693,7 +2707,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2708,7 +2722,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -2717,7 +2731,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2741,7 +2755,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2756,7 +2770,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2765,7 +2779,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2780,11 +2794,35 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F50" s="27" t="n"/>
       <c r="G50" s="27" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F51" s="27" t="n"/>
+      <c r="G51" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates + 1 account event (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-23 05:24 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-23 10:15 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -995,9 +995,11 @@
         <v>18461</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H6" s="22" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>387</v>
+      </c>
       <c r="I6" s="22" t="n"/>
       <c r="J6" s="22" t="n"/>
       <c r="K6" s="23" t="n"/>
@@ -1397,7 +1399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1455,101 +1457,115 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>9097</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
       <c r="G2" s="27" t="n"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="G3" s="27" t="n"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
-      <c r="G4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G4" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1559,11 +1575,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>10808</v>
+        <v>9097</v>
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
@@ -1575,43 +1591,31 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n"/>
       <c r="G6" s="27" t="n"/>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1626,7 +1630,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F7" s="27" t="n"/>
@@ -1635,129 +1639,127 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G8" s="27" t="n"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G9" s="27" t="n"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n"/>
       <c r="G10" s="27" t="n"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G11" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1781,7 +1783,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1796,26 +1798,38 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1829,9 +1843,11 @@
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>4842</v>
-      </c>
-      <c r="G14" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>app</t>
@@ -1841,7 +1857,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1865,82 +1881,82 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
       <c r="G16" s="27" t="n"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G17" s="27" t="n"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
@@ -1949,17 +1965,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1969,38 +1985,38 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>12641</v>
+        <v>0</v>
       </c>
       <c r="G19" s="27" t="n"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F20" s="27" t="n"/>
@@ -2009,77 +2025,77 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
       <c r="G21" s="27" t="n"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G22" s="27" t="n"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2093,17 +2109,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2113,15 +2129,13 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G24" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>5345</v>
+      </c>
+      <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>app</t>
@@ -2131,17 +2145,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2155,17 +2169,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2179,17 +2193,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2199,13 +2213,15 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>10383</v>
-      </c>
-      <c r="G27" s="27" t="n"/>
+        <v>1985</v>
+      </c>
+      <c r="G27" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>app</t>
@@ -2215,22 +2231,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2239,17 +2255,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2263,17 +2279,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2283,11 +2299,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>100</v>
+        <v>10383</v>
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
@@ -2299,58 +2315,46 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
       <c r="G31" s="27" t="n"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2359,106 +2363,118 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G33" s="27" t="n"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
       <c r="G35" s="27" t="n"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F36" s="27" t="n"/>
@@ -2467,17 +2483,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2491,41 +2507,53 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G38" s="27" t="n"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2539,7 +2567,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2554,7 +2582,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F40" s="27" t="n"/>
@@ -2563,7 +2591,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2578,7 +2606,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F41" s="27" t="n"/>
@@ -2587,7 +2615,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2611,22 +2639,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F43" s="27" t="n"/>
@@ -2635,22 +2663,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2659,22 +2687,22 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2683,7 +2711,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2707,7 +2735,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2722,7 +2750,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -2731,7 +2759,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2746,7 +2774,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F48" s="27" t="n"/>
@@ -2755,7 +2783,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2779,7 +2807,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2794,7 +2822,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F50" s="27" t="n"/>
@@ -2803,7 +2831,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2818,11 +2846,83 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F51" s="27" t="n"/>
       <c r="G51" s="27" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F52" s="27" t="n"/>
+      <c r="G52" s="27" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F53" s="27" t="n"/>
+      <c r="G53" s="27" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F54" s="27" t="n"/>
+      <c r="G54" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates (luis, eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-23 15:06 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-23 19:06 UTC by the Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -998,7 +998,7 @@
         <v>9720</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>831</v>
+        <v>2650</v>
       </c>
       <c r="I6" s="22" t="n"/>
       <c r="J6" s="22" t="n"/>
@@ -1091,7 +1091,9 @@
       <c r="G8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="22" t="n"/>
+      <c r="H8" s="22" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="22" t="n"/>
       <c r="J8" s="22" t="n"/>
       <c r="K8" s="23" t="n"/>
@@ -1399,7 +1401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1457,7 +1459,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1481,10 +1483,10 @@
         </is>
       </c>
       <c r="F2" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G2" s="27" t="n">
         <v>831</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>387</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1495,31 +1497,43 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G3" s="27" t="n"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1543,9 +1557,11 @@
         </is>
       </c>
       <c r="F4" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G4" s="27" t="n">
         <v>387</v>
       </c>
-      <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>app</t>
@@ -1555,7 +1571,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1570,40 +1586,26 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1613,11 +1615,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>9097</v>
+        <v>387</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
@@ -1629,190 +1631,216 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G8" s="27" t="n"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
       <c r="G9" s="27" t="n"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n"/>
       <c r="G10" s="27" t="n"/>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G11" s="27" t="n"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G12" s="27" t="n"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F13" s="27" t="n"/>
@@ -1821,43 +1849,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n"/>
       <c r="G14" s="27" t="n"/>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1872,30 +1888,16 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G15" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1910,16 +1912,28 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G16" s="27" t="n"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1934,52 +1948,54 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
       <c r="G18" s="27" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1994,7 +2010,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F19" s="27" t="n"/>
@@ -2003,17 +2019,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2027,34 +2043,34 @@
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="G20" s="27" t="n"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F21" s="27" t="n"/>
@@ -2063,67 +2079,67 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G22" s="27" t="n"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2138,7 +2154,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2147,17 +2163,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2171,7 +2187,7 @@
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>5345</v>
+        <v>12641</v>
       </c>
       <c r="G25" s="27" t="n"/>
       <c r="H25" t="inlineStr">
@@ -2183,22 +2199,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F26" s="27" t="n"/>
@@ -2207,7 +2223,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2222,69 +2238,67 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G27" s="27" t="n"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G28" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F29" s="27" t="n"/>
@@ -2293,82 +2307,84 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n"/>
-      <c r="G30" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G30" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
       <c r="G31" s="27" t="n"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2377,7 +2393,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2392,136 +2408,148 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G33" s="27" t="n"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
       <c r="G34" s="27" t="n"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
       <c r="G35" s="27" t="n"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G36" s="27" t="n"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G37" s="27" t="n"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2536,7 +2564,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F38" s="27" t="n"/>
@@ -2545,53 +2573,41 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F39" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="n"/>
       <c r="G39" s="27" t="n"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2605,46 +2621,58 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G41" s="27" t="n"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2653,7 +2681,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2677,7 +2705,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2701,7 +2729,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2716,7 +2744,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2725,7 +2753,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2740,7 +2768,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F46" s="27" t="n"/>
@@ -2749,22 +2777,22 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -2773,22 +2801,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F48" s="27" t="n"/>
@@ -2797,7 +2825,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2812,7 +2840,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2821,7 +2849,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2845,7 +2873,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2869,7 +2897,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2893,7 +2921,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2908,7 +2936,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -2917,7 +2945,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2932,7 +2960,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F54" s="27" t="n"/>
@@ -2941,7 +2969,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2956,11 +2984,59 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
       <c r="G55" s="27" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n"/>
+      <c r="G56" s="27" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F57" s="27" t="n"/>
+      <c r="G57" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 4 step updates (luis)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-23 19:06 UTC by the Team 8 app</t>
+          <t>Updated 2026-10-23 19:56 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1084,15 +1084,17 @@
         <f>SUM(E8:AE8)</f>
         <v/>
       </c>
-      <c r="E8" s="22" t="n"/>
+      <c r="E8" s="22" t="n">
+        <v>4933</v>
+      </c>
       <c r="F8" s="22" t="n">
-        <v>0</v>
+        <v>7567</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>0</v>
+        <v>4189</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>0</v>
+        <v>3685</v>
       </c>
       <c r="I8" s="22" t="n"/>
       <c r="J8" s="22" t="n"/>
@@ -1401,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1459,17 +1461,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1479,15 +1481,13 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>831</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>app</t>
@@ -1497,7 +1497,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1517,33 +1517,35 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F3" s="27" t="n">
+        <v>7567</v>
+      </c>
+      <c r="G3" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="27" t="n"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1553,14 +1555,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>831</v>
+        <v>4189</v>
       </c>
       <c r="G4" s="27" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1571,31 +1573,45 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n"/>
-      <c r="G5" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1619,9 +1635,11 @@
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>387</v>
-      </c>
-      <c r="G6" s="27" t="n"/>
+        <v>2650</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>app</t>
@@ -1631,17 +1649,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1651,35 +1669,33 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>1100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1689,13 +1705,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G8" s="27" t="n"/>
+        <v>831</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>app</t>
@@ -1705,22 +1723,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -1729,41 +1747,53 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="G10" s="27" t="n"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1773,13 +1803,15 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>10808</v>
-      </c>
-      <c r="G11" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>app</t>
@@ -1789,17 +1821,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1813,19 +1845,19 @@
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>0</v>
+        <v>9097</v>
       </c>
       <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1849,7 +1881,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1873,41 +1905,53 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G15" s="27" t="n"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1921,72 +1965,58 @@
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G17" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
+      <c r="G17" s="27" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F18" s="27" t="n"/>
@@ -1995,7 +2025,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2010,7 +2040,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F19" s="27" t="n"/>
@@ -2019,17 +2049,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2039,11 +2069,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>4842</v>
+        <v>1100</v>
       </c>
       <c r="G20" s="27" t="n"/>
       <c r="H20" t="inlineStr">
@@ -2055,7 +2085,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2070,67 +2100,69 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n"/>
-      <c r="G21" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n"/>
       <c r="G22" s="27" t="n"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F23" s="27" t="n"/>
@@ -2139,137 +2171,137 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G24" s="27" t="n"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
       <c r="G25" s="27" t="n"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G26" s="27" t="n"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n"/>
       <c r="G27" s="27" t="n"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2283,108 +2315,118 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G29" s="27" t="n"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G30" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n"/>
+      <c r="G30" s="27" t="n"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G31" s="27" t="n"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2393,82 +2435,84 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n"/>
       <c r="G33" s="27" t="n"/>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
-      <c r="G34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G34" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F35" s="27" t="n"/>
@@ -2477,53 +2521,41 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n"/>
       <c r="G36" s="27" t="n"/>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2537,7 +2569,7 @@
         </is>
       </c>
       <c r="F37" s="27" t="n">
-        <v>9060</v>
+        <v>10383</v>
       </c>
       <c r="G37" s="27" t="n"/>
       <c r="H37" t="inlineStr">
@@ -2549,17 +2581,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2573,22 +2605,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2597,41 +2629,53 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F40" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G40" s="27" t="n"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2645,7 +2689,7 @@
         </is>
       </c>
       <c r="F41" s="27" t="n">
-        <v>6310</v>
+        <v>9060</v>
       </c>
       <c r="G41" s="27" t="n"/>
       <c r="H41" t="inlineStr">
@@ -2657,22 +2701,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2681,22 +2725,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F43" s="27" t="n"/>
@@ -2705,22 +2749,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2729,46 +2773,58 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F45" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G45" s="27" t="n"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F46" s="27" t="n"/>
@@ -2777,7 +2833,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2792,7 +2848,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -2801,7 +2857,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2816,7 +2872,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F48" s="27" t="n"/>
@@ -2825,22 +2881,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2849,22 +2905,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F50" s="27" t="n"/>
@@ -2873,22 +2929,22 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F51" s="27" t="n"/>
@@ -2897,22 +2953,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F52" s="27" t="n"/>
@@ -2921,7 +2977,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2936,7 +2992,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -2945,7 +3001,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2969,7 +3025,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2984,7 +3040,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
@@ -2993,7 +3049,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3008,7 +3064,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F56" s="27" t="n"/>
@@ -3017,7 +3073,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3032,11 +3088,107 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F57" s="27" t="n"/>
       <c r="G57" s="27" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F58" s="27" t="n"/>
+      <c r="G58" s="27" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n"/>
+      <c r="G59" s="27" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F60" s="27" t="n"/>
+      <c r="G60" s="27" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F61" s="27" t="n"/>
+      <c r="G61" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update + 1 story (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-23 22:03 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-24 04:52 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -998,7 +998,7 @@
         <v>9720</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>2680</v>
+        <v>8981</v>
       </c>
       <c r="I6" s="22" t="n"/>
       <c r="J6" s="22" t="n"/>
@@ -1403,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1461,7 +1461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1485,10 +1485,10 @@
         </is>
       </c>
       <c r="F2" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G2" s="27" t="n">
         <v>2680</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>2650</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -1499,53 +1499,41 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n">
-        <v>4933</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
       <c r="G3" s="27" t="n"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1555,14 +1543,14 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>7567</v>
+        <v>2680</v>
       </c>
       <c r="G4" s="27" t="n">
-        <v>0</v>
+        <v>2650</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1573,7 +1561,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1593,15 +1581,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>4189</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>app</t>
@@ -1611,7 +1597,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1631,35 +1617,35 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>3685</v>
+        <v>7567</v>
       </c>
       <c r="G6" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1669,14 +1655,14 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>2650</v>
+        <v>4189</v>
       </c>
       <c r="G7" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1687,7 +1673,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1711,9 +1697,11 @@
         </is>
       </c>
       <c r="F8" s="27" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G8" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>shortcut</t>
@@ -1723,7 +1711,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1747,10 +1735,10 @@
         </is>
       </c>
       <c r="F9" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G9" s="27" t="n">
         <v>831</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>387</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1761,31 +1749,43 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G10" s="27" t="n"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1809,9 +1809,11 @@
         </is>
       </c>
       <c r="F11" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G11" s="27" t="n">
         <v>387</v>
       </c>
-      <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>app</t>
@@ -1821,7 +1823,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1836,40 +1838,26 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n"/>
+      <c r="G12" s="27" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1879,11 +1867,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>9097</v>
+        <v>387</v>
       </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" t="inlineStr">
@@ -1895,190 +1883,216 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G15" s="27" t="n"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
       <c r="G16" s="27" t="n"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
       <c r="G17" s="27" t="n"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G18" s="27" t="n"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G19" s="27" t="n"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F20" s="27" t="n"/>
@@ -2087,43 +2101,31 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
       <c r="G21" s="27" t="n"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2138,30 +2140,16 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G22" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="n"/>
+      <c r="G22" s="27" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2176,16 +2164,28 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G23" s="27" t="n"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2200,52 +2200,54 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n"/>
-      <c r="G24" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G24" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
       <c r="G25" s="27" t="n"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2260,7 +2262,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F26" s="27" t="n"/>
@@ -2269,17 +2271,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2293,34 +2295,34 @@
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="G27" s="27" t="n"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2329,67 +2331,67 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G29" s="27" t="n"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n"/>
       <c r="G30" s="27" t="n"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2404,7 +2406,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F31" s="27" t="n"/>
@@ -2413,17 +2415,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2437,7 +2439,7 @@
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>5345</v>
+        <v>12641</v>
       </c>
       <c r="G32" s="27" t="n"/>
       <c r="H32" t="inlineStr">
@@ -2449,22 +2451,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F33" s="27" t="n"/>
@@ -2473,7 +2475,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2488,69 +2490,67 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G35" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
+      <c r="G35" s="27" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F36" s="27" t="n"/>
@@ -2559,82 +2559,84 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n"/>
-      <c r="G37" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G37" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n"/>
       <c r="G38" s="27" t="n"/>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2643,7 +2645,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2658,136 +2660,148 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F40" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G40" s="27" t="n"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="n"/>
       <c r="G41" s="27" t="n"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n"/>
       <c r="G42" s="27" t="n"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G43" s="27" t="n"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G44" s="27" t="n"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2802,7 +2816,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2811,53 +2825,41 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n"/>
       <c r="G46" s="27" t="n"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2871,46 +2873,58 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G48" s="27" t="n"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2919,7 +2933,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2943,7 +2957,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2967,7 +2981,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2982,7 +2996,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F52" s="27" t="n"/>
@@ -2991,7 +3005,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3006,7 +3020,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -3015,22 +3029,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F54" s="27" t="n"/>
@@ -3039,22 +3053,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
@@ -3063,7 +3077,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3078,7 +3092,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F56" s="27" t="n"/>
@@ -3087,7 +3101,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3111,7 +3125,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3135,7 +3149,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3159,7 +3173,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3174,7 +3188,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F60" s="27" t="n"/>
@@ -3183,7 +3197,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3198,7 +3212,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3207,7 +3221,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3222,11 +3236,59 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F62" s="27" t="n"/>
       <c r="G62" s="27" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="n"/>
+      <c r="G63" s="27" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F64" s="27" t="n"/>
+      <c r="G64" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update (luis)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-24 18:58 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-25 01:22 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1098,7 +1098,9 @@
       <c r="H8" s="22" t="n">
         <v>3685</v>
       </c>
-      <c r="I8" s="22" t="n"/>
+      <c r="I8" s="22" t="n">
+        <v>7493</v>
+      </c>
       <c r="J8" s="22" t="n"/>
       <c r="K8" s="23" t="n"/>
       <c r="L8" s="23" t="n"/>
@@ -1405,7 +1407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1463,17 +1465,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1487,21 +1489,19 @@
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1525,10 +1525,10 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
+        <v>122</v>
+      </c>
+      <c r="G3" s="27" t="n">
         <v>121</v>
-      </c>
-      <c r="G3" s="27" t="n">
-        <v>120</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1539,7 +1539,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1563,9 +1563,11 @@
         </is>
       </c>
       <c r="F4" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G4" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>app</t>
@@ -1575,7 +1577,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1595,15 +1597,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>app</t>
@@ -1613,7 +1613,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1628,16 +1628,30 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n"/>
-      <c r="G6" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1652,40 +1666,26 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1695,13 +1695,15 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G8" s="27" t="n"/>
+        <v>2680</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>2650</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>app</t>
@@ -1711,7 +1713,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1731,15 +1733,13 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>app</t>
@@ -1749,7 +1749,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>4189</v>
+        <v>7567</v>
       </c>
       <c r="G10" s="27" t="n">
         <v>0</v>
@@ -1787,7 +1787,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1807,35 +1807,35 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>3685</v>
+        <v>4189</v>
       </c>
       <c r="G11" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1849,31 +1849,31 @@
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>2650</v>
+        <v>3685</v>
       </c>
       <c r="G12" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1887,29 +1887,31 @@
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="27" t="n"/>
+        <v>2650</v>
+      </c>
+      <c r="G13" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1923,21 +1925,19 @@
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>387</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G14" s="27" t="n"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1952,16 +1952,30 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>387</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1976,28 +1990,16 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
-        <v>387</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n"/>
       <c r="G16" s="27" t="n"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2017,15 +2019,13 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G17" s="27" t="n">
-        <v>1100</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="G17" s="27" t="n"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>app</t>
@@ -2035,17 +2035,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2059,9 +2059,11 @@
         </is>
       </c>
       <c r="F18" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G18" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G18" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>app</t>
@@ -2071,31 +2073,43 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G19" s="27" t="n"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2110,7 +2124,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F20" s="27" t="n"/>
@@ -2119,53 +2133,41 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n"/>
       <c r="G21" s="27" t="n"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2175,47 +2177,59 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>0</v>
+        <v>10808</v>
       </c>
       <c r="G22" s="27" t="n"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G23" s="27" t="n"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2230,7 +2244,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F24" s="27" t="n"/>
@@ -2239,22 +2253,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F25" s="27" t="n"/>
@@ -2263,7 +2277,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2278,28 +2292,16 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n"/>
       <c r="G26" s="27" t="n"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2319,15 +2321,13 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G27" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G27" s="27" t="n"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>app</t>
@@ -2337,7 +2337,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2352,16 +2352,30 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n"/>
-      <c r="G28" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G28" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2376,7 +2390,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F29" s="27" t="n"/>
@@ -2385,103 +2399,91 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n"/>
       <c r="G30" s="27" t="n"/>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G31" s="27" t="n"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="n"/>
       <c r="G32" s="27" t="n"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2496,31 +2498,43 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G33" s="27" t="n"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F34" s="27" t="n"/>
@@ -2529,7 +2543,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2544,28 +2558,16 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
       <c r="G35" s="27" t="n"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2580,52 +2582,52 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G36" s="27" t="n"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
       <c r="G37" s="27" t="n"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2640,16 +2642,28 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G38" s="27" t="n"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2664,7 +2678,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2673,69 +2687,69 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F40" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G40" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G41" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2750,7 +2764,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2759,43 +2773,31 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n"/>
       <c r="G43" s="27" t="n"/>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2810,16 +2812,28 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G44" s="27" t="n"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2834,7 +2848,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2843,43 +2857,31 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n"/>
       <c r="G46" s="27" t="n"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2899,11 +2901,11 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F47" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G47" s="27" t="n"/>
       <c r="H47" t="inlineStr">
@@ -2915,31 +2917,43 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G48" s="27" t="n"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2954,7 +2968,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2963,7 +2977,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2978,7 +2992,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F50" s="27" t="n"/>
@@ -2987,43 +3001,31 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F51" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F51" s="27" t="n"/>
       <c r="G51" s="27" t="n"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3038,26 +3040,38 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F52" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F52" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G52" s="27" t="n"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3071,7 +3085,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3086,7 +3100,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F54" s="27" t="n"/>
@@ -3095,7 +3109,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3110,7 +3124,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
@@ -3119,7 +3133,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3134,7 +3148,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F56" s="27" t="n"/>
@@ -3143,7 +3157,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3158,7 +3172,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F57" s="27" t="n"/>
@@ -3167,7 +3181,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3182,7 +3196,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F58" s="27" t="n"/>
@@ -3191,22 +3205,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F59" s="27" t="n"/>
@@ -3215,7 +3229,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3239,7 +3253,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3254,7 +3268,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3263,7 +3277,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3278,7 +3292,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F62" s="27" t="n"/>
@@ -3287,7 +3301,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3302,7 +3316,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F63" s="27" t="n"/>
@@ -3311,7 +3325,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3326,7 +3340,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F64" s="27" t="n"/>
@@ -3335,7 +3349,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3359,7 +3373,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3374,7 +3388,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F66" s="27" t="n"/>
@@ -3383,7 +3397,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3398,11 +3412,35 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F67" s="27" t="n"/>
       <c r="G67" s="27" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F68" s="27" t="n"/>
+      <c r="G68" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 story (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-25 06:17 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-25 15:02 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1407,7 +1407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H69"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1465,7 +1465,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1480,40 +1480,26 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1527,29 +1513,31 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G3" s="27" t="n"/>
+        <v>8060</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>122</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1563,21 +1551,19 @@
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G4" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1601,10 +1587,10 @@
         </is>
       </c>
       <c r="F5" s="27" t="n">
+        <v>122</v>
+      </c>
+      <c r="G5" s="27" t="n">
         <v>121</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>120</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1615,7 +1601,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1639,9 +1625,11 @@
         </is>
       </c>
       <c r="F6" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G6" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>app</t>
@@ -1651,7 +1639,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1671,15 +1659,13 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>app</t>
@@ -1689,7 +1675,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1704,16 +1690,30 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
-      <c r="G8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1728,40 +1728,26 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1771,13 +1757,15 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G10" s="27" t="n"/>
+        <v>2680</v>
+      </c>
+      <c r="G10" s="27" t="n">
+        <v>2650</v>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
           <t>app</t>
@@ -1787,7 +1775,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1807,15 +1795,13 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G11" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>app</t>
@@ -1825,7 +1811,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1845,11 +1831,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>4189</v>
+        <v>7567</v>
       </c>
       <c r="G12" s="27" t="n">
         <v>0</v>
@@ -1863,7 +1849,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1883,35 +1869,35 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>3685</v>
+        <v>4189</v>
       </c>
       <c r="G13" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1925,31 +1911,31 @@
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>2650</v>
+        <v>3685</v>
       </c>
       <c r="G14" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1963,29 +1949,31 @@
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="27" t="n"/>
+        <v>2650</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1999,21 +1987,19 @@
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>387</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2028,16 +2014,30 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n"/>
-      <c r="G17" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>387</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2052,28 +2052,16 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>387</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
       <c r="G18" s="27" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2093,15 +2081,13 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G19" s="27" t="n">
-        <v>1100</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="G19" s="27" t="n"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>app</t>
@@ -2111,17 +2097,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2135,9 +2121,11 @@
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G20" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>app</t>
@@ -2147,31 +2135,43 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G21" s="27" t="n"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F22" s="27" t="n"/>
@@ -2195,53 +2195,41 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2251,47 +2239,59 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>0</v>
+        <v>10808</v>
       </c>
       <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G25" s="27" t="n"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2306,7 +2306,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F26" s="27" t="n"/>
@@ -2315,22 +2315,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F27" s="27" t="n"/>
@@ -2339,7 +2339,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2354,28 +2354,16 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n"/>
       <c r="G28" s="27" t="n"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2395,15 +2383,13 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F29" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G29" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G29" s="27" t="n"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>app</t>
@@ -2413,7 +2399,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2428,16 +2414,30 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n"/>
-      <c r="G30" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G30" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F31" s="27" t="n"/>
@@ -2461,103 +2461,91 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="n"/>
       <c r="G32" s="27" t="n"/>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G33" s="27" t="n"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
       <c r="G34" s="27" t="n"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2572,31 +2560,43 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G35" s="27" t="n"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F36" s="27" t="n"/>
@@ -2605,7 +2605,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2620,28 +2620,16 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
       <c r="G37" s="27" t="n"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2656,52 +2644,52 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G38" s="27" t="n"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F39" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="n"/>
       <c r="G39" s="27" t="n"/>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2716,16 +2704,28 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F40" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F40" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G40" s="27" t="n"/>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2740,7 +2740,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F41" s="27" t="n"/>
@@ -2749,69 +2749,69 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G42" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n"/>
+      <c r="G42" s="27" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n"/>
-      <c r="G43" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G43" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F44" s="27" t="n"/>
@@ -2835,43 +2835,31 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F45" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="n"/>
       <c r="G45" s="27" t="n"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2886,16 +2874,28 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G46" s="27" t="n"/>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2910,7 +2910,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -2919,43 +2919,31 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n"/>
       <c r="G48" s="27" t="n"/>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2975,11 +2963,11 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G49" s="27" t="n"/>
       <c r="H49" t="inlineStr">
@@ -2991,31 +2979,43 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F50" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F50" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G50" s="27" t="n"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F51" s="27" t="n"/>
@@ -3039,7 +3039,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F52" s="27" t="n"/>
@@ -3063,43 +3063,31 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F53" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F53" s="27" t="n"/>
       <c r="G53" s="27" t="n"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3114,26 +3102,38 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F54" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F54" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G54" s="27" t="n"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3147,7 +3147,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F56" s="27" t="n"/>
@@ -3171,7 +3171,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F57" s="27" t="n"/>
@@ -3195,7 +3195,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F58" s="27" t="n"/>
@@ -3219,7 +3219,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3234,7 +3234,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F59" s="27" t="n"/>
@@ -3243,7 +3243,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F60" s="27" t="n"/>
@@ -3267,22 +3267,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3291,7 +3291,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3315,7 +3315,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F63" s="27" t="n"/>
@@ -3339,7 +3339,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F64" s="27" t="n"/>
@@ -3363,7 +3363,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F65" s="27" t="n"/>
@@ -3387,7 +3387,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F66" s="27" t="n"/>
@@ -3411,7 +3411,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F68" s="27" t="n"/>
@@ -3459,7 +3459,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3474,11 +3474,35 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F69" s="27" t="n"/>
       <c r="G69" s="27" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F70" s="27" t="n"/>
+      <c r="G70" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 3 step updates (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-26 01:02 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-26 05:57 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1004,9 +1004,11 @@
         <v>8060</v>
       </c>
       <c r="J6" s="22" t="n">
+        <v>20274</v>
+      </c>
+      <c r="K6" s="23" t="n">
         <v>351</v>
       </c>
-      <c r="K6" s="23" t="n"/>
       <c r="L6" s="23" t="n"/>
       <c r="M6" s="23" t="n"/>
       <c r="N6" s="23" t="n"/>
@@ -1411,7 +1413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1469,17 +1471,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1489,23 +1491,23 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>13001</v>
+        <v>351</v>
       </c>
       <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1529,9 +1531,11 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>351</v>
-      </c>
-      <c r="G3" s="27" t="n"/>
+        <v>20274</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>3510</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>app</t>
@@ -1541,7 +1545,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1556,26 +1560,40 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
-      <c r="G4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G4" s="27" t="n">
+        <v>351</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1585,35 +1603,33 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>122</v>
-      </c>
+        <v>13001</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1623,23 +1639,23 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>7493</v>
+        <v>351</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1654,30 +1670,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>121</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1701,10 +1703,10 @@
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>121</v>
+        <v>8060</v>
       </c>
       <c r="G8" s="27" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1715,17 +1717,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1739,19 +1741,19 @@
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>120</v>
+        <v>7493</v>
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1771,14 +1773,14 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>8981</v>
+        <v>122</v>
       </c>
       <c r="G10" s="27" t="n">
-        <v>2680</v>
+        <v>121</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1789,7 +1791,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1804,16 +1806,30 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n"/>
-      <c r="G11" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>120</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1833,15 +1849,13 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>2650</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>app</t>
@@ -1851,17 +1865,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1871,13 +1885,15 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G13" s="27" t="n"/>
+        <v>8981</v>
+      </c>
+      <c r="G13" s="27" t="n">
+        <v>2680</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>app</t>
@@ -1887,55 +1903,41 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n"/>
+      <c r="G14" s="27" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1945,14 +1947,14 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>4189</v>
+        <v>2680</v>
       </c>
       <c r="G15" s="27" t="n">
-        <v>0</v>
+        <v>2650</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1963,7 +1965,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1983,35 +1985,33 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>3685</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2021,14 +2021,14 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>2650</v>
+        <v>7567</v>
       </c>
       <c r="G17" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2039,7 +2039,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2059,33 +2059,35 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F18" s="27" t="n">
+        <v>4189</v>
+      </c>
+      <c r="G18" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="27" t="n"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2099,21 +2101,21 @@
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>831</v>
+        <v>3685</v>
       </c>
       <c r="G19" s="27" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2128,26 +2130,40 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n"/>
-      <c r="G20" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2161,19 +2177,19 @@
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="G21" s="27" t="n"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2193,14 +2209,14 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>9720</v>
+        <v>831</v>
       </c>
       <c r="G22" s="27" t="n">
-        <v>1100</v>
+        <v>387</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2211,101 +2227,115 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>9097</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="G24" s="27" t="n"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n"/>
-      <c r="G25" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G25" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2315,11 +2345,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>10808</v>
+        <v>9097</v>
       </c>
       <c r="G26" s="27" t="n"/>
       <c r="H26" t="inlineStr">
@@ -2331,43 +2361,31 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n"/>
       <c r="G27" s="27" t="n"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2382,7 +2400,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2391,129 +2409,127 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G29" s="27" t="n"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G30" s="27" t="n"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
       <c r="G31" s="27" t="n"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G32" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="n"/>
+      <c r="G32" s="27" t="n"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2537,7 +2553,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2552,26 +2568,38 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2585,9 +2613,11 @@
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>4842</v>
-      </c>
-      <c r="G35" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G35" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
           <t>app</t>
@@ -2597,7 +2627,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2621,82 +2651,82 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
       <c r="G37" s="27" t="n"/>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G38" s="27" t="n"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2705,17 +2735,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2725,38 +2755,38 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
-        <v>12641</v>
+        <v>0</v>
       </c>
       <c r="G40" s="27" t="n"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F41" s="27" t="n"/>
@@ -2765,77 +2795,77 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n"/>
       <c r="G42" s="27" t="n"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G43" s="27" t="n"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2849,17 +2879,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2869,15 +2899,13 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F45" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G45" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>5345</v>
+      </c>
+      <c r="G45" s="27" t="n"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>app</t>
@@ -2887,17 +2915,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2911,17 +2939,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2935,17 +2963,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2955,13 +2983,15 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F48" s="27" t="n">
-        <v>10383</v>
-      </c>
-      <c r="G48" s="27" t="n"/>
+        <v>1985</v>
+      </c>
+      <c r="G48" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>app</t>
@@ -2971,22 +3001,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -2995,17 +3025,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3019,17 +3049,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3039,11 +3069,11 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F51" s="27" t="n">
-        <v>100</v>
+        <v>10383</v>
       </c>
       <c r="G51" s="27" t="n"/>
       <c r="H51" t="inlineStr">
@@ -3055,58 +3085,46 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F52" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F52" s="27" t="n"/>
       <c r="G52" s="27" t="n"/>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -3115,106 +3133,118 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F54" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F54" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G54" s="27" t="n"/>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F55" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F55" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G55" s="27" t="n"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n"/>
       <c r="G56" s="27" t="n"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F57" s="27" t="n"/>
@@ -3223,17 +3253,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3247,41 +3277,53 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G59" s="27" t="n"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3295,7 +3337,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3310,7 +3352,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3319,7 +3361,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3334,7 +3376,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F62" s="27" t="n"/>
@@ -3343,7 +3385,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3367,22 +3409,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F64" s="27" t="n"/>
@@ -3391,22 +3433,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F65" s="27" t="n"/>
@@ -3415,22 +3457,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F66" s="27" t="n"/>
@@ -3439,7 +3481,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3463,7 +3505,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3478,7 +3520,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F68" s="27" t="n"/>
@@ -3487,7 +3529,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3502,7 +3544,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F69" s="27" t="n"/>
@@ -3511,7 +3553,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3535,7 +3577,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3550,7 +3592,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F71" s="27" t="n"/>
@@ -3559,7 +3601,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3574,11 +3616,83 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F72" s="27" t="n"/>
       <c r="G72" s="27" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F73" s="27" t="n"/>
+      <c r="G73" s="27" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F74" s="27" t="n"/>
+      <c r="G74" s="27" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F75" s="27" t="n"/>
+      <c r="G75" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates + 1 story (luis, eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-26 18:39 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-27 01:38 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1007,7 +1007,7 @@
         <v>20274</v>
       </c>
       <c r="K6" s="23" t="n">
-        <v>911</v>
+        <v>1157</v>
       </c>
       <c r="L6" s="23" t="n"/>
       <c r="M6" s="23" t="n"/>
@@ -1108,7 +1108,9 @@
       <c r="J8" s="22" t="n">
         <v>13001</v>
       </c>
-      <c r="K8" s="23" t="n"/>
+      <c r="K8" s="23" t="n">
+        <v>8300</v>
+      </c>
       <c r="L8" s="23" t="n"/>
       <c r="M8" s="23" t="n"/>
       <c r="N8" s="23" t="n"/>
@@ -1413,7 +1415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1471,7 +1473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1486,30 +1488,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>351</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1533,9 +1521,11 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>351</v>
-      </c>
-      <c r="G3" s="27" t="n"/>
+        <v>1157</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>911</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>app</t>
@@ -1545,17 +1535,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1565,25 +1555,23 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G4" s="27" t="n">
-        <v>3510</v>
-      </c>
+        <v>8300</v>
+      </c>
+      <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1603,11 +1591,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>3510</v>
+        <v>911</v>
       </c>
       <c r="G5" s="27" t="n">
         <v>351</v>
@@ -1621,17 +1609,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1641,23 +1629,23 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>13001</v>
+        <v>351</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1681,9 +1669,11 @@
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>351</v>
-      </c>
-      <c r="G7" s="27" t="n"/>
+        <v>20274</v>
+      </c>
+      <c r="G7" s="27" t="n">
+        <v>3510</v>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>app</t>
@@ -1693,7 +1683,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1708,26 +1698,40 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
-      <c r="G8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>351</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1737,35 +1741,33 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>122</v>
-      </c>
+        <v>13001</v>
+      </c>
+      <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1775,23 +1777,23 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>7493</v>
+        <v>351</v>
       </c>
       <c r="G10" s="27" t="n"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1806,30 +1808,16 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G11" s="27" t="n">
-        <v>121</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="27" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1853,10 +1841,10 @@
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>121</v>
+        <v>8060</v>
       </c>
       <c r="G12" s="27" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1867,17 +1855,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1891,19 +1879,19 @@
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>120</v>
+        <v>7493</v>
       </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1923,14 +1911,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>8981</v>
+        <v>122</v>
       </c>
       <c r="G14" s="27" t="n">
-        <v>2680</v>
+        <v>121</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1941,7 +1929,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1956,16 +1944,30 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>120</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1985,15 +1987,13 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>2650</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>app</t>
@@ -2003,17 +2003,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2023,13 +2023,15 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G17" s="27" t="n"/>
+        <v>8981</v>
+      </c>
+      <c r="G17" s="27" t="n">
+        <v>2680</v>
+      </c>
       <c r="H17" t="inlineStr">
         <is>
           <t>app</t>
@@ -2039,55 +2041,41 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G18" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2097,14 +2085,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>4189</v>
+        <v>2680</v>
       </c>
       <c r="G19" s="27" t="n">
-        <v>0</v>
+        <v>2650</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2115,7 +2103,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2135,35 +2123,33 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>3685</v>
-      </c>
-      <c r="G20" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G20" s="27" t="n"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2173,14 +2159,14 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>2650</v>
+        <v>7567</v>
       </c>
       <c r="G21" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2191,7 +2177,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2211,33 +2197,35 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
+        <v>4189</v>
+      </c>
+      <c r="G22" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="27" t="n"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2251,21 +2239,21 @@
         </is>
       </c>
       <c r="F23" s="27" t="n">
-        <v>831</v>
+        <v>3685</v>
       </c>
       <c r="G23" s="27" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2280,26 +2268,40 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n"/>
-      <c r="G24" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G24" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2313,19 +2315,19 @@
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="G25" s="27" t="n"/>
       <c r="H25" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2345,14 +2347,14 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>9720</v>
+        <v>831</v>
       </c>
       <c r="G26" s="27" t="n">
-        <v>1100</v>
+        <v>387</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2363,101 +2365,115 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n">
-        <v>9097</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n"/>
       <c r="G27" s="27" t="n"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="G28" s="27" t="n"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n"/>
-      <c r="G29" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G29" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2467,11 +2483,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>10808</v>
+        <v>9097</v>
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
@@ -2483,43 +2499,31 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
       <c r="G31" s="27" t="n"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2534,7 +2538,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F32" s="27" t="n"/>
@@ -2543,129 +2547,127 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G33" s="27" t="n"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n"/>
       <c r="G35" s="27" t="n"/>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G36" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2689,7 +2691,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2704,26 +2706,38 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G38" s="27" t="n"/>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2737,9 +2751,11 @@
         </is>
       </c>
       <c r="F39" s="27" t="n">
-        <v>4842</v>
-      </c>
-      <c r="G39" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G39" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>app</t>
@@ -2749,7 +2765,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2773,82 +2789,82 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="n"/>
       <c r="G41" s="27" t="n"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G42" s="27" t="n"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F43" s="27" t="n"/>
@@ -2857,17 +2873,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2877,38 +2893,38 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F44" s="27" t="n">
-        <v>12641</v>
+        <v>0</v>
       </c>
       <c r="G44" s="27" t="n"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F45" s="27" t="n"/>
@@ -2917,77 +2933,77 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n"/>
       <c r="G46" s="27" t="n"/>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F47" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F47" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G47" s="27" t="n"/>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3001,17 +3017,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3021,15 +3037,13 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G49" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>5345</v>
+      </c>
+      <c r="G49" s="27" t="n"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>app</t>
@@ -3039,17 +3053,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3063,17 +3077,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3087,17 +3101,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3107,13 +3121,15 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F52" s="27" t="n">
-        <v>10383</v>
-      </c>
-      <c r="G52" s="27" t="n"/>
+        <v>1985</v>
+      </c>
+      <c r="G52" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
           <t>app</t>
@@ -3123,22 +3139,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -3147,17 +3163,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3171,17 +3187,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3191,11 +3207,11 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F55" s="27" t="n">
-        <v>100</v>
+        <v>10383</v>
       </c>
       <c r="G55" s="27" t="n"/>
       <c r="H55" t="inlineStr">
@@ -3207,58 +3223,46 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n"/>
       <c r="G56" s="27" t="n"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F57" s="27" t="n"/>
@@ -3267,106 +3271,118 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F58" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F58" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G58" s="27" t="n"/>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G59" s="27" t="n"/>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F60" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F60" s="27" t="n"/>
       <c r="G60" s="27" t="n"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3375,17 +3391,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3399,41 +3415,53 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F63" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G63" s="27" t="n"/>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3447,7 +3475,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3462,7 +3490,7 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F65" s="27" t="n"/>
@@ -3471,7 +3499,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3486,7 +3514,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F66" s="27" t="n"/>
@@ -3495,7 +3523,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3519,22 +3547,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F68" s="27" t="n"/>
@@ -3543,22 +3571,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F69" s="27" t="n"/>
@@ -3567,22 +3595,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F70" s="27" t="n"/>
@@ -3591,7 +3619,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3615,7 +3643,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3630,7 +3658,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F72" s="27" t="n"/>
@@ -3639,7 +3667,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3654,7 +3682,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F73" s="27" t="n"/>
@@ -3663,7 +3691,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3687,7 +3715,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3702,7 +3730,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F75" s="27" t="n"/>
@@ -3711,7 +3739,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3726,11 +3754,83 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F76" s="27" t="n"/>
       <c r="G76" s="27" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F77" s="27" t="n"/>
+      <c r="G77" s="27" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F78" s="27" t="n"/>
+      <c r="G78" s="27" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F79" s="27" t="n"/>
+      <c r="G79" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 5 step updates (armando, eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-27 12:43 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-27 18:18 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1010,7 +1010,7 @@
         <v>15809</v>
       </c>
       <c r="L6" s="23" t="n">
-        <v>311</v>
+        <v>1401</v>
       </c>
       <c r="M6" s="23" t="n"/>
       <c r="N6" s="23" t="n"/>
@@ -1203,10 +1203,18 @@
       <c r="G10" s="22" t="n">
         <v>9097</v>
       </c>
-      <c r="H10" s="22" t="n"/>
-      <c r="I10" s="22" t="n"/>
-      <c r="J10" s="22" t="n"/>
-      <c r="K10" s="23" t="n"/>
+      <c r="H10" s="22" t="n">
+        <v>4947</v>
+      </c>
+      <c r="I10" s="22" t="n">
+        <v>3787</v>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>307</v>
+      </c>
+      <c r="K10" s="23" t="n">
+        <v>4640</v>
+      </c>
       <c r="L10" s="23" t="n"/>
       <c r="M10" s="23" t="n"/>
       <c r="N10" s="23" t="n"/>
@@ -1417,7 +1425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1475,7 +1483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1499,9 +1507,11 @@
         </is>
       </c>
       <c r="F2" s="27" t="n">
+        <v>1401</v>
+      </c>
+      <c r="G2" s="27" t="n">
         <v>311</v>
       </c>
-      <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>app</t>
@@ -1511,17 +1521,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1535,11 +1545,9 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G3" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>4640</v>
+      </c>
+      <c r="G3" s="27" t="n"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>app</t>
@@ -1549,41 +1557,53 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>307</v>
+      </c>
       <c r="G4" s="27" t="n"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1593,15 +1613,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>1157</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>911</v>
-      </c>
+        <v>3787</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>app</t>
@@ -1611,17 +1629,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1631,23 +1649,23 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>8300</v>
+        <v>4947</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1667,15 +1685,13 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>app</t>
@@ -1685,7 +1701,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1709,9 +1725,11 @@
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>351</v>
-      </c>
-      <c r="G8" s="27" t="n"/>
+        <v>15809</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>1157</v>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>app</t>
@@ -1721,7 +1739,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1736,30 +1754,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>3510</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n"/>
+      <c r="G9" s="27" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1779,14 +1783,14 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>3510</v>
+        <v>1157</v>
       </c>
       <c r="G10" s="27" t="n">
-        <v>351</v>
+        <v>911</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1797,7 +1801,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1817,11 +1821,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>13001</v>
+        <v>8300</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
@@ -1833,7 +1837,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1853,13 +1857,15 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
+        <v>911</v>
+      </c>
+      <c r="G12" s="27" t="n">
         <v>351</v>
       </c>
-      <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>app</t>
@@ -1869,7 +1875,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1884,16 +1890,28 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1913,14 +1931,14 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>8060</v>
+        <v>20274</v>
       </c>
       <c r="G14" s="27" t="n">
-        <v>122</v>
+        <v>3510</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1931,17 +1949,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1951,33 +1969,35 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G15" s="27" t="n"/>
+        <v>3510</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1987,25 +2007,23 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G16" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>13001</v>
+      </c>
+      <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2025,15 +2043,13 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>121</v>
-      </c>
-      <c r="G17" s="27" t="n">
-        <v>120</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G17" s="27" t="n"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>app</t>
@@ -2043,7 +2059,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2058,28 +2074,16 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>120</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
       <c r="G18" s="27" t="n"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2099,14 +2103,14 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>8981</v>
+        <v>8060</v>
       </c>
       <c r="G19" s="27" t="n">
-        <v>2680</v>
+        <v>122</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2117,31 +2121,43 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n">
+        <v>7493</v>
+      </c>
       <c r="G20" s="27" t="n"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2161,14 +2177,14 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>2680</v>
+        <v>122</v>
       </c>
       <c r="G21" s="27" t="n">
-        <v>2650</v>
+        <v>121</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2179,17 +2195,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2199,13 +2215,15 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G22" s="27" t="n"/>
+        <v>121</v>
+      </c>
+      <c r="G22" s="27" t="n">
+        <v>120</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>app</t>
@@ -2215,17 +2233,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2235,15 +2253,13 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F23" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G23" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G23" s="27" t="n"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>app</t>
@@ -2253,17 +2269,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2273,14 +2289,14 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>4189</v>
+        <v>8981</v>
       </c>
       <c r="G24" s="27" t="n">
-        <v>0</v>
+        <v>2680</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -2291,45 +2307,31 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>3685</v>
-      </c>
-      <c r="G25" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n"/>
+      <c r="G25" s="27" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2353,10 +2355,10 @@
         </is>
       </c>
       <c r="F26" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G26" s="27" t="n">
         <v>2650</v>
-      </c>
-      <c r="G26" s="27" t="n">
-        <v>831</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2367,7 +2369,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2387,33 +2389,33 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>0</v>
+        <v>4933</v>
       </c>
       <c r="G27" s="27" t="n"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2423,14 +2425,14 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F28" s="27" t="n">
-        <v>831</v>
+        <v>7567</v>
       </c>
       <c r="G28" s="27" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -2441,41 +2443,55 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n"/>
-      <c r="G29" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n">
+        <v>4189</v>
+      </c>
+      <c r="G29" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2489,19 +2505,21 @@
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>387</v>
-      </c>
-      <c r="G30" s="27" t="n"/>
+        <v>3685</v>
+      </c>
+      <c r="G30" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2521,14 +2539,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F31" s="27" t="n">
-        <v>9720</v>
+        <v>2650</v>
       </c>
       <c r="G31" s="27" t="n">
-        <v>1100</v>
+        <v>831</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -2539,17 +2557,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2559,62 +2577,76 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>9097</v>
+        <v>0</v>
       </c>
       <c r="G32" s="27" t="n"/>
       <c r="H32" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n"/>
-      <c r="G33" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G33" s="27" t="n">
+        <v>387</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F34" s="27" t="n"/>
@@ -2623,17 +2655,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2643,11 +2675,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>10808</v>
+        <v>387</v>
       </c>
       <c r="G35" s="27" t="n"/>
       <c r="H35" t="inlineStr">
@@ -2659,17 +2691,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2683,43 +2715,57 @@
         </is>
       </c>
       <c r="F36" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G36" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G37" s="27" t="n"/>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2734,7 +2780,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F38" s="27" t="n"/>
@@ -2743,22 +2789,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F39" s="27" t="n"/>
@@ -2767,17 +2813,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2787,11 +2833,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
-        <v>1100</v>
+        <v>10808</v>
       </c>
       <c r="G40" s="27" t="n"/>
       <c r="H40" t="inlineStr">
@@ -2803,17 +2849,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2823,40 +2869,38 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F41" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G41" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G41" s="27" t="n"/>
       <c r="H41" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2865,22 +2909,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F43" s="27" t="n"/>
@@ -2889,43 +2933,31 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n"/>
       <c r="G44" s="27" t="n"/>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2940,26 +2972,38 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F45" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G45" s="27" t="n"/>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2973,34 +3017,36 @@
         </is>
       </c>
       <c r="F46" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G46" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -3009,22 +3055,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F48" s="27" t="n"/>
@@ -3033,17 +3079,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3053,11 +3099,11 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>12641</v>
+        <v>4842</v>
       </c>
       <c r="G49" s="27" t="n"/>
       <c r="H49" t="inlineStr">
@@ -3069,22 +3115,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F50" s="27" t="n"/>
@@ -3093,17 +3139,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3113,38 +3159,38 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F51" s="27" t="n">
-        <v>5345</v>
+        <v>0</v>
       </c>
       <c r="G51" s="27" t="n"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F52" s="27" t="n"/>
@@ -3153,22 +3199,22 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -3177,17 +3223,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3197,15 +3243,13 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F54" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G54" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>12641</v>
+      </c>
+      <c r="G54" s="27" t="n"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>app</t>
@@ -3215,22 +3259,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
@@ -3239,82 +3283,82 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G56" s="27" t="n"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F57" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F57" s="27" t="n"/>
       <c r="G57" s="27" t="n"/>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F58" s="27" t="n"/>
@@ -3323,142 +3367,144 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n"/>
-      <c r="G59" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G59" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F60" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F60" s="27" t="n"/>
       <c r="G60" s="27" t="n"/>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F61" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F61" s="27" t="n"/>
       <c r="G61" s="27" t="n"/>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F62" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F62" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G62" s="27" t="n"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F63" s="27" t="n"/>
@@ -3467,17 +3513,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3491,17 +3537,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3511,11 +3557,11 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F65" s="27" t="n">
-        <v>6310</v>
+        <v>100</v>
       </c>
       <c r="G65" s="27" t="n"/>
       <c r="H65" t="inlineStr">
@@ -3527,46 +3573,58 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F66" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F66" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G66" s="27" t="n"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F67" s="27" t="n"/>
@@ -3575,22 +3633,22 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F68" s="27" t="n"/>
@@ -3599,17 +3657,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3623,46 +3681,58 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F70" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F70" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G70" s="27" t="n"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F71" s="27" t="n"/>
@@ -3671,7 +3741,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3695,22 +3765,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F73" s="27" t="n"/>
@@ -3719,22 +3789,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F74" s="27" t="n"/>
@@ -3743,22 +3813,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F75" s="27" t="n"/>
@@ -3767,22 +3837,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F76" s="27" t="n"/>
@@ -3791,22 +3861,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F77" s="27" t="n"/>
@@ -3815,7 +3885,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3839,7 +3909,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3863,7 +3933,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3878,7 +3948,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -3887,7 +3957,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3902,11 +3972,131 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F81" s="27" t="n"/>
       <c r="G81" s="27" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F82" s="27" t="n"/>
+      <c r="G82" s="27" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F83" s="27" t="n"/>
+      <c r="G83" s="27" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F84" s="27" t="n"/>
+      <c r="G84" s="27" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F85" s="27" t="n"/>
+      <c r="G85" s="27" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F86" s="27" t="n"/>
+      <c r="G86" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 8 step updates (minerva, eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-27 18:18 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-28 07:03 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1010,9 +1010,11 @@
         <v>15809</v>
       </c>
       <c r="L6" s="23" t="n">
-        <v>1401</v>
-      </c>
-      <c r="M6" s="23" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="M6" s="23" t="n">
+        <v>271</v>
+      </c>
       <c r="N6" s="23" t="n"/>
       <c r="O6" s="23" t="n"/>
       <c r="P6" s="23" t="n"/>
@@ -1258,12 +1260,24 @@
       <c r="F11" s="22" t="n">
         <v>10808</v>
       </c>
-      <c r="G11" s="22" t="n"/>
-      <c r="H11" s="22" t="n"/>
-      <c r="I11" s="22" t="n"/>
-      <c r="J11" s="22" t="n"/>
-      <c r="K11" s="23" t="n"/>
-      <c r="L11" s="23" t="n"/>
+      <c r="G11" s="22" t="n">
+        <v>13681</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>11109</v>
+      </c>
+      <c r="I11" s="22" t="n">
+        <v>10595</v>
+      </c>
+      <c r="J11" s="22" t="n">
+        <v>10320</v>
+      </c>
+      <c r="K11" s="23" t="n">
+        <v>10300</v>
+      </c>
+      <c r="L11" s="23" t="n">
+        <v>12221</v>
+      </c>
       <c r="M11" s="23" t="n"/>
       <c r="N11" s="23" t="n"/>
       <c r="O11" s="23" t="n"/>
@@ -1425,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1483,7 +1497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27 15:27:47</t>
+          <t>2026-10-28 06:27:01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1503,15 +1517,13 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>311</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>app</t>
@@ -1521,17 +1533,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-27 14:45:13</t>
+          <t>2026-10-28 06:26:50</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1541,13 +1553,15 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>4640</v>
-      </c>
-      <c r="G3" s="27" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>1401</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>app</t>
@@ -1557,17 +1571,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:39</t>
+          <t>2026-10-28 05:23:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1581,7 +1595,7 @@
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>307</v>
+        <v>10320</v>
       </c>
       <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
@@ -1593,17 +1607,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:05</t>
+          <t>2026-10-28 05:21:45</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1613,11 +1627,11 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>3787</v>
+        <v>12221</v>
       </c>
       <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
@@ -1629,17 +1643,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-27 14:41:31</t>
+          <t>2026-10-28 05:20:41</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1649,11 +1663,11 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>4947</v>
+        <v>10300</v>
       </c>
       <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
@@ -1665,17 +1679,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-28 05:15:21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1685,11 +1699,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>311</v>
+        <v>10595</v>
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
@@ -1701,17 +1715,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-28 05:13:25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1721,15 +1735,13 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G8" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>11109</v>
+      </c>
+      <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>app</t>
@@ -1739,31 +1751,43 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-28 05:12:16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="n">
+        <v>13681</v>
+      </c>
       <c r="G9" s="27" t="n"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1783,14 +1807,14 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>1157</v>
+        <v>1401</v>
       </c>
       <c r="G10" s="27" t="n">
-        <v>911</v>
+        <v>311</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1801,17 +1825,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1825,29 +1849,29 @@
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>8300</v>
+        <v>4640</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1857,15 +1881,13 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>307</v>
+      </c>
+      <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>app</t>
@@ -1875,17 +1897,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1895,11 +1917,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>351</v>
+        <v>3787</v>
       </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" t="inlineStr">
@@ -1911,17 +1933,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1931,15 +1953,13 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G14" s="27" t="n">
-        <v>3510</v>
-      </c>
+        <v>4947</v>
+      </c>
+      <c r="G14" s="27" t="n"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>app</t>
@@ -1949,7 +1969,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1969,15 +1989,13 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>3510</v>
-      </c>
-      <c r="G15" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G15" s="27" t="n"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>app</t>
@@ -1987,17 +2005,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2007,23 +2025,25 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>13001</v>
-      </c>
-      <c r="G16" s="27" t="n"/>
+        <v>15809</v>
+      </c>
+      <c r="G16" s="27" t="n">
+        <v>1157</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2038,28 +2058,16 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
-        <v>351</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="n"/>
       <c r="G17" s="27" t="n"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2074,26 +2082,40 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n"/>
-      <c r="G18" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="G18" s="27" t="n">
+        <v>911</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2103,35 +2125,33 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G19" s="27" t="n">
-        <v>122</v>
-      </c>
+        <v>8300</v>
+      </c>
+      <c r="G19" s="27" t="n"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2141,23 +2161,25 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G20" s="27" t="n"/>
+        <v>911</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2177,15 +2199,13 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G21" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G21" s="27" t="n"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>app</t>
@@ -2195,7 +2215,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2215,14 +2235,14 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>121</v>
+        <v>20274</v>
       </c>
       <c r="G22" s="27" t="n">
-        <v>120</v>
+        <v>3510</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2233,7 +2253,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2253,13 +2273,15 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F23" s="27" t="n">
-        <v>120</v>
-      </c>
-      <c r="G23" s="27" t="n"/>
+        <v>3510</v>
+      </c>
+      <c r="G23" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>app</t>
@@ -2269,17 +2291,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2289,25 +2311,23 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G24" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>13001</v>
+      </c>
+      <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2322,16 +2342,28 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="G25" s="27" t="n"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2346,40 +2378,26 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G26" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="27" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2389,13 +2407,15 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G27" s="27" t="n"/>
+        <v>8060</v>
+      </c>
+      <c r="G27" s="27" t="n">
+        <v>122</v>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>app</t>
@@ -2405,7 +2425,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2425,35 +2445,33 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F28" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G28" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G28" s="27" t="n"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2463,14 +2481,14 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F29" s="27" t="n">
-        <v>4189</v>
+        <v>122</v>
       </c>
       <c r="G29" s="27" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -2481,17 +2499,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2501,25 +2519,25 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>3685</v>
+        <v>121</v>
       </c>
       <c r="G30" s="27" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2539,15 +2557,13 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F31" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="G31" s="27" t="n">
-        <v>831</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G31" s="27" t="n"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>app</t>
@@ -2557,17 +2573,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2581,19 +2597,21 @@
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="27" t="n"/>
+        <v>8981</v>
+      </c>
+      <c r="G32" s="27" t="n">
+        <v>2680</v>
+      </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2608,30 +2626,16 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G33" s="27" t="n">
-        <v>387</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="n"/>
+      <c r="G33" s="27" t="n"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2646,26 +2650,40 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
-      <c r="G34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G34" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2675,11 +2693,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>387</v>
+        <v>4933</v>
       </c>
       <c r="G35" s="27" t="n"/>
       <c r="H35" t="inlineStr">
@@ -2691,17 +2709,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2711,14 +2729,14 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F36" s="27" t="n">
-        <v>9720</v>
+        <v>7567</v>
       </c>
       <c r="G36" s="27" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2729,17 +2747,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2753,9 +2771,11 @@
         </is>
       </c>
       <c r="F37" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G37" s="27" t="n"/>
+        <v>4189</v>
+      </c>
+      <c r="G37" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>app</t>
@@ -2765,65 +2785,93 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n"/>
-      <c r="G38" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F38" s="27" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G38" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F39" s="27" t="n"/>
-      <c r="G39" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F39" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G39" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2833,33 +2881,33 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
-        <v>10808</v>
+        <v>0</v>
       </c>
       <c r="G40" s="27" t="n"/>
       <c r="H40" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2869,38 +2917,40 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F41" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="27" t="n"/>
+        <v>831</v>
+      </c>
+      <c r="G41" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F42" s="27" t="n"/>
@@ -2909,31 +2959,43 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="G43" s="27" t="n"/>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2948,26 +3010,40 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n"/>
-      <c r="G44" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G44" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2981,7 +3057,7 @@
         </is>
       </c>
       <c r="F45" s="27" t="n">
-        <v>1100</v>
+        <v>9097</v>
       </c>
       <c r="G45" s="27" t="n"/>
       <c r="H45" t="inlineStr">
@@ -2993,60 +3069,46 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G46" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n"/>
+      <c r="G46" s="27" t="n"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F47" s="27" t="n"/>
@@ -3055,41 +3117,53 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G48" s="27" t="n"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3099,38 +3173,38 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>4842</v>
+        <v>0</v>
       </c>
       <c r="G49" s="27" t="n"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F50" s="27" t="n"/>
@@ -3139,58 +3213,46 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F51" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F51" s="27" t="n"/>
       <c r="G51" s="27" t="n"/>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F52" s="27" t="n"/>
@@ -3199,41 +3261,53 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F53" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F53" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G53" s="27" t="n"/>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3243,13 +3317,15 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F54" s="27" t="n">
-        <v>12641</v>
-      </c>
-      <c r="G54" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G54" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>app</t>
@@ -3259,22 +3335,22 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F55" s="27" t="n"/>
@@ -3283,43 +3359,31 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n"/>
       <c r="G56" s="27" t="n"/>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3334,31 +3398,43 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F57" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F57" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G57" s="27" t="n"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F58" s="27" t="n"/>
@@ -3367,17 +3443,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3391,36 +3467,34 @@
         </is>
       </c>
       <c r="F59" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G59" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G59" s="27" t="n"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F60" s="27" t="n"/>
@@ -3429,22 +3503,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3453,17 +3527,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3477,7 +3551,7 @@
         </is>
       </c>
       <c r="F62" s="27" t="n">
-        <v>10383</v>
+        <v>12641</v>
       </c>
       <c r="G62" s="27" t="n"/>
       <c r="H62" t="inlineStr">
@@ -3489,22 +3563,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F63" s="27" t="n"/>
@@ -3513,137 +3587,139 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F64" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F64" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G64" s="27" t="n"/>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F65" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F65" s="27" t="n"/>
       <c r="G65" s="27" t="n"/>
-      <c r="H65" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F66" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F66" s="27" t="n"/>
       <c r="G66" s="27" t="n"/>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F67" s="27" t="n"/>
-      <c r="G67" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F67" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G67" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3657,17 +3733,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3681,17 +3757,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3705,7 +3781,7 @@
         </is>
       </c>
       <c r="F70" s="27" t="n">
-        <v>6310</v>
+        <v>10383</v>
       </c>
       <c r="G70" s="27" t="n"/>
       <c r="H70" t="inlineStr">
@@ -3717,22 +3793,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F71" s="27" t="n"/>
@@ -3741,17 +3817,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3765,70 +3841,94 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F73" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G73" s="27" t="n"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F74" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F74" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G74" s="27" t="n"/>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F75" s="27" t="n"/>
@@ -3837,22 +3937,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F76" s="27" t="n"/>
@@ -3861,17 +3961,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3885,46 +3985,58 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F78" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F78" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G78" s="27" t="n"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F79" s="27" t="n"/>
@@ -3933,22 +4045,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -3957,22 +4069,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F81" s="27" t="n"/>
@@ -3981,22 +4093,22 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F82" s="27" t="n"/>
@@ -4005,22 +4117,22 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F83" s="27" t="n"/>
@@ -4029,22 +4141,22 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F84" s="27" t="n"/>
@@ -4053,22 +4165,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F85" s="27" t="n"/>
@@ -4077,7 +4189,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4092,11 +4204,203 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
       <c r="G86" s="27" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:41:34</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F87" s="27" t="n"/>
+      <c r="G87" s="27" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:41:28</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="n"/>
+      <c r="G88" s="27" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:27:02</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="n"/>
+      <c r="G89" s="27" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="n"/>
+      <c r="G90" s="27" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F91" s="27" t="n"/>
+      <c r="G91" s="27" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F92" s="27" t="n"/>
+      <c r="G92" s="27" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F93" s="27" t="n"/>
+      <c r="G93" s="27" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F94" s="27" t="n"/>
+      <c r="G94" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 account event (eron)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-28 19:15 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-28 21:28 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1439,7 +1439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H96"/>
+  <dimension ref="A1:H97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1497,7 +1497,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-28 17:45:48</t>
+          <t>2026-10-28 21:24:32</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1512,30 +1512,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>371</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>271</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-28 10:22:51</t>
+          <t>2026-10-28 17:45:48</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1550,16 +1536,30 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n"/>
-      <c r="G3" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>271</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-28 06:27:01</t>
+          <t>2026-10-28 10:22:51</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1574,28 +1574,16 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n">
-        <v>271</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n"/>
       <c r="G4" s="27" t="n"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-28 06:26:50</t>
+          <t>2026-10-28 06:27:01</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1615,15 +1603,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>9670</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>1401</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>app</t>
@@ -1633,17 +1619,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-28 05:23:00</t>
+          <t>2026-10-28 06:26:50</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1653,13 +1639,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>10320</v>
-      </c>
-      <c r="G6" s="27" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>1401</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>app</t>
@@ -1669,7 +1657,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-28 05:21:45</t>
+          <t>2026-10-28 05:23:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1689,11 +1677,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>12221</v>
+        <v>10320</v>
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
@@ -1705,7 +1693,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-28 05:20:41</t>
+          <t>2026-10-28 05:21:45</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1725,11 +1713,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>10300</v>
+        <v>12221</v>
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
@@ -1741,7 +1729,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-28 05:15:21</t>
+          <t>2026-10-28 05:20:41</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1761,11 +1749,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>10595</v>
+        <v>10300</v>
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
@@ -1777,7 +1765,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-28 05:13:25</t>
+          <t>2026-10-28 05:15:21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1797,11 +1785,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>11109</v>
+        <v>10595</v>
       </c>
       <c r="G10" s="27" t="n"/>
       <c r="H10" t="inlineStr">
@@ -1813,7 +1801,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-28 05:12:16</t>
+          <t>2026-10-28 05:13:25</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1833,11 +1821,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>13681</v>
+        <v>11109</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
@@ -1849,17 +1837,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-27 15:27:47</t>
+          <t>2026-10-28 05:12:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1869,15 +1857,13 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>311</v>
-      </c>
+        <v>13681</v>
+      </c>
+      <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>app</t>
@@ -1887,17 +1873,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-27 14:45:13</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1907,13 +1893,15 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>4640</v>
-      </c>
-      <c r="G13" s="27" t="n"/>
+        <v>1401</v>
+      </c>
+      <c r="G13" s="27" t="n">
+        <v>311</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>app</t>
@@ -1923,7 +1911,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:39</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1943,11 +1931,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>307</v>
+        <v>4640</v>
       </c>
       <c r="G14" s="27" t="n"/>
       <c r="H14" t="inlineStr">
@@ -1959,7 +1947,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:05</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1979,11 +1967,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>3787</v>
+        <v>307</v>
       </c>
       <c r="G15" s="27" t="n"/>
       <c r="H15" t="inlineStr">
@@ -1995,7 +1983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-27 14:41:31</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2015,11 +2003,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>4947</v>
+        <v>3787</v>
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
@@ -2031,17 +2019,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2051,11 +2039,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>311</v>
+        <v>4947</v>
       </c>
       <c r="G17" s="27" t="n"/>
       <c r="H17" t="inlineStr">
@@ -2067,7 +2055,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2087,15 +2075,13 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F18" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G18" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G18" s="27" t="n"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>app</t>
@@ -2105,7 +2091,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2120,16 +2106,30 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n"/>
-      <c r="G19" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="n">
+        <v>15809</v>
+      </c>
+      <c r="G19" s="27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2144,40 +2144,26 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n">
-        <v>1157</v>
-      </c>
-      <c r="G20" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="n"/>
+      <c r="G20" s="27" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2191,29 +2177,31 @@
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>8300</v>
-      </c>
-      <c r="G21" s="27" t="n"/>
+        <v>1157</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <v>911</v>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2227,21 +2215,19 @@
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G22" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>8300</v>
+      </c>
+      <c r="G22" s="27" t="n"/>
       <c r="H22" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2265,9 +2251,11 @@
         </is>
       </c>
       <c r="F23" s="27" t="n">
+        <v>911</v>
+      </c>
+      <c r="G23" s="27" t="n">
         <v>351</v>
       </c>
-      <c r="G23" s="27" t="n"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>app</t>
@@ -2277,7 +2265,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2297,15 +2285,13 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G24" s="27" t="n">
-        <v>3510</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>app</t>
@@ -2315,7 +2301,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2339,10 +2325,10 @@
         </is>
       </c>
       <c r="F25" s="27" t="n">
+        <v>20274</v>
+      </c>
+      <c r="G25" s="27" t="n">
         <v>3510</v>
-      </c>
-      <c r="G25" s="27" t="n">
-        <v>351</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2353,17 +2339,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2377,29 +2363,31 @@
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>13001</v>
-      </c>
-      <c r="G26" s="27" t="n"/>
+        <v>3510</v>
+      </c>
+      <c r="G26" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2413,19 +2401,19 @@
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>351</v>
+        <v>13001</v>
       </c>
       <c r="G27" s="27" t="n"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2440,16 +2428,28 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="G28" s="27" t="n"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2464,40 +2464,26 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G29" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n"/>
+      <c r="G29" s="27" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2511,29 +2497,31 @@
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G30" s="27" t="n"/>
+        <v>8060</v>
+      </c>
+      <c r="G30" s="27" t="n">
+        <v>122</v>
+      </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2547,21 +2535,19 @@
         </is>
       </c>
       <c r="F31" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G31" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G31" s="27" t="n"/>
       <c r="H31" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2585,10 +2571,10 @@
         </is>
       </c>
       <c r="F32" s="27" t="n">
+        <v>122</v>
+      </c>
+      <c r="G32" s="27" t="n">
         <v>121</v>
-      </c>
-      <c r="G32" s="27" t="n">
-        <v>120</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -2599,7 +2585,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2623,9 +2609,11 @@
         </is>
       </c>
       <c r="F33" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G33" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="G33" s="27" t="n"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>app</t>
@@ -2635,7 +2623,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2655,15 +2643,13 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G34" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G34" s="27" t="n"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>app</t>
@@ -2673,7 +2659,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2688,16 +2674,30 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n"/>
-      <c r="G35" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F35" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G35" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2712,40 +2712,26 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G36" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n"/>
+      <c r="G36" s="27" t="n"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2755,13 +2741,15 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F37" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G37" s="27" t="n"/>
+        <v>2680</v>
+      </c>
+      <c r="G37" s="27" t="n">
+        <v>2650</v>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>app</t>
@@ -2771,7 +2759,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2791,15 +2779,13 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F38" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G38" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G38" s="27" t="n"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>app</t>
@@ -2809,7 +2795,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2829,11 +2815,11 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F39" s="27" t="n">
-        <v>4189</v>
+        <v>7567</v>
       </c>
       <c r="G39" s="27" t="n">
         <v>0</v>
@@ -2847,7 +2833,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2867,35 +2853,35 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
-        <v>3685</v>
+        <v>4189</v>
       </c>
       <c r="G40" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2909,31 +2895,31 @@
         </is>
       </c>
       <c r="F41" s="27" t="n">
-        <v>2650</v>
+        <v>3685</v>
       </c>
       <c r="G41" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2947,29 +2933,31 @@
         </is>
       </c>
       <c r="F42" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="27" t="n"/>
+        <v>2650</v>
+      </c>
+      <c r="G42" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2983,21 +2971,19 @@
         </is>
       </c>
       <c r="F43" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G43" s="27" t="n">
-        <v>387</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G43" s="27" t="n"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3012,16 +2998,30 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n"/>
-      <c r="G44" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G44" s="27" t="n">
+        <v>387</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3036,28 +3036,16 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F45" s="27" t="n">
-        <v>387</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F45" s="27" t="n"/>
       <c r="G45" s="27" t="n"/>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3077,15 +3065,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F46" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G46" s="27" t="n">
-        <v>1100</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="G46" s="27" t="n"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>app</t>
@@ -3095,17 +3081,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3119,9 +3105,11 @@
         </is>
       </c>
       <c r="F47" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G47" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G47" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H47" t="inlineStr">
         <is>
           <t>app</t>
@@ -3131,31 +3119,43 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G48" s="27" t="n"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F49" s="27" t="n"/>
@@ -3179,53 +3179,41 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F50" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F50" s="27" t="n"/>
       <c r="G50" s="27" t="n"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3235,47 +3223,59 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F51" s="27" t="n">
-        <v>0</v>
+        <v>10808</v>
       </c>
       <c r="G51" s="27" t="n"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F52" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F52" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G52" s="27" t="n"/>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F53" s="27" t="n"/>
@@ -3299,22 +3299,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F54" s="27" t="n"/>
@@ -3323,7 +3323,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3338,28 +3338,16 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F55" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F55" s="27" t="n"/>
       <c r="G55" s="27" t="n"/>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3379,15 +3367,13 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F56" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G56" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G56" s="27" t="n"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>app</t>
@@ -3397,7 +3383,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3412,16 +3398,30 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F57" s="27" t="n"/>
-      <c r="G57" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F57" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G57" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3436,7 +3436,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F58" s="27" t="n"/>
@@ -3445,103 +3445,91 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n"/>
       <c r="G59" s="27" t="n"/>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F60" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F60" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G60" s="27" t="n"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F61" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F61" s="27" t="n"/>
       <c r="G61" s="27" t="n"/>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3556,31 +3544,43 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F62" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F62" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G62" s="27" t="n"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F63" s="27" t="n"/>
@@ -3589,7 +3589,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3604,28 +3604,16 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F64" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F64" s="27" t="n"/>
       <c r="G64" s="27" t="n"/>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3640,52 +3628,52 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F65" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F65" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G65" s="27" t="n"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F66" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F66" s="27" t="n"/>
       <c r="G66" s="27" t="n"/>
-      <c r="H66" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3700,16 +3688,28 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F67" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F67" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G67" s="27" t="n"/>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F68" s="27" t="n"/>
@@ -3733,69 +3733,69 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F69" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G69" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F69" s="27" t="n"/>
+      <c r="G69" s="27" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F70" s="27" t="n"/>
-      <c r="G70" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F70" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G70" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3810,7 +3810,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F71" s="27" t="n"/>
@@ -3819,43 +3819,31 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F72" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F72" s="27" t="n"/>
       <c r="G72" s="27" t="n"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3870,16 +3858,28 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F73" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G73" s="27" t="n"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F74" s="27" t="n"/>
@@ -3903,43 +3903,31 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F75" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F75" s="27" t="n"/>
       <c r="G75" s="27" t="n"/>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3959,11 +3947,11 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F76" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G76" s="27" t="n"/>
       <c r="H76" t="inlineStr">
@@ -3975,31 +3963,43 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F77" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F77" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G77" s="27" t="n"/>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F78" s="27" t="n"/>
@@ -4023,7 +4023,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F79" s="27" t="n"/>
@@ -4047,43 +4047,31 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F80" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F80" s="27" t="n"/>
       <c r="G80" s="27" t="n"/>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4098,26 +4086,38 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F81" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F81" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G81" s="27" t="n"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4131,7 +4131,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F83" s="27" t="n"/>
@@ -4155,7 +4155,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F84" s="27" t="n"/>
@@ -4179,7 +4179,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F85" s="27" t="n"/>
@@ -4203,7 +4203,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
@@ -4227,7 +4227,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4242,7 +4242,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F87" s="27" t="n"/>
@@ -4251,22 +4251,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F88" s="27" t="n"/>
@@ -4275,7 +4275,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4299,7 +4299,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4314,7 +4314,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F90" s="27" t="n"/>
@@ -4323,7 +4323,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F91" s="27" t="n"/>
@@ -4347,7 +4347,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4362,7 +4362,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F92" s="27" t="n"/>
@@ -4371,7 +4371,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F93" s="27" t="n"/>
@@ -4395,7 +4395,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4419,7 +4419,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F95" s="27" t="n"/>
@@ -4443,7 +4443,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4458,11 +4458,35 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F96" s="27" t="n"/>
       <c r="G96" s="27" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F97" s="27" t="n"/>
+      <c r="G97" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 step update (minerva)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-29 14:45 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-29 14:51 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1284,7 +1284,9 @@
       <c r="L11" s="23" t="n">
         <v>12221</v>
       </c>
-      <c r="M11" s="23" t="n"/>
+      <c r="M11" s="23" t="n">
+        <v>10100</v>
+      </c>
       <c r="N11" s="23" t="n"/>
       <c r="O11" s="23" t="n"/>
       <c r="P11" s="23" t="n"/>
@@ -1445,7 +1447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1503,17 +1505,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-29 14:44:19</t>
+          <t>2026-10-29 14:50:59</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1523,15 +1525,13 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>1011</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>266</v>
-      </c>
+        <v>10100</v>
+      </c>
+      <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>app</t>
@@ -1541,17 +1541,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-29 09:14:12</t>
+          <t>2026-10-29 14:44:19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1565,29 +1565,31 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>30</v>
-      </c>
-      <c r="G3" s="27" t="n"/>
+        <v>1011</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>266</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-29 06:32:56</t>
+          <t>2026-10-29 09:14:12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1601,19 +1603,19 @@
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>266</v>
+        <v>30</v>
       </c>
       <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-29 02:35:57</t>
+          <t>2026-10-29 06:32:56</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1633,15 +1635,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>21456</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>2371</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>app</t>
@@ -1651,17 +1651,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-29 00:00:12</t>
+          <t>2026-10-29 02:35:57</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1675,29 +1675,31 @@
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>4018</v>
-      </c>
-      <c r="G6" s="27" t="n"/>
+        <v>21456</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>2371</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-28 23:47:44</t>
+          <t>2026-10-29 00:00:12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1711,21 +1713,19 @@
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>2371</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>371</v>
-      </c>
+        <v>4018</v>
+      </c>
+      <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-28 23:46:44</t>
+          <t>2026-10-28 23:47:44</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1740,16 +1740,30 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n"/>
-      <c r="G8" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>2371</v>
+      </c>
+      <c r="G8" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-28 21:24:32</t>
+          <t>2026-10-28 23:46:44</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1764,7 +1778,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F9" s="27" t="n"/>
@@ -1773,7 +1787,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-28 17:45:48</t>
+          <t>2026-10-28 21:24:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1788,30 +1802,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n">
-        <v>371</v>
-      </c>
-      <c r="G10" s="27" t="n">
-        <v>271</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="n"/>
+      <c r="G10" s="27" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-28 10:22:51</t>
+          <t>2026-10-28 17:45:48</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1826,16 +1826,30 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n"/>
-      <c r="G11" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="G11" s="27" t="n">
+        <v>271</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-28 06:27:01</t>
+          <t>2026-10-28 10:22:51</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1850,28 +1864,16 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n">
-        <v>271</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="n"/>
       <c r="G12" s="27" t="n"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-28 06:26:50</t>
+          <t>2026-10-28 06:27:01</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1891,15 +1893,13 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>9670</v>
-      </c>
-      <c r="G13" s="27" t="n">
-        <v>1401</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="G13" s="27" t="n"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>app</t>
@@ -1909,17 +1909,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-28 05:23:00</t>
+          <t>2026-10-28 06:26:50</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1929,13 +1929,15 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>10320</v>
-      </c>
-      <c r="G14" s="27" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>1401</v>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>app</t>
@@ -1945,7 +1947,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-28 05:21:45</t>
+          <t>2026-10-28 05:23:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1965,11 +1967,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>12221</v>
+        <v>10320</v>
       </c>
       <c r="G15" s="27" t="n"/>
       <c r="H15" t="inlineStr">
@@ -1981,7 +1983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-28 05:20:41</t>
+          <t>2026-10-28 05:21:45</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2001,11 +2003,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>10300</v>
+        <v>12221</v>
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
@@ -2017,7 +2019,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-28 05:15:21</t>
+          <t>2026-10-28 05:20:41</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2037,11 +2039,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>10595</v>
+        <v>10300</v>
       </c>
       <c r="G17" s="27" t="n"/>
       <c r="H17" t="inlineStr">
@@ -2053,7 +2055,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-28 05:13:25</t>
+          <t>2026-10-28 05:15:21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2073,11 +2075,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F18" s="27" t="n">
-        <v>11109</v>
+        <v>10595</v>
       </c>
       <c r="G18" s="27" t="n"/>
       <c r="H18" t="inlineStr">
@@ -2089,7 +2091,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-28 05:12:16</t>
+          <t>2026-10-28 05:13:25</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2109,11 +2111,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>13681</v>
+        <v>11109</v>
       </c>
       <c r="G19" s="27" t="n"/>
       <c r="H19" t="inlineStr">
@@ -2125,17 +2127,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-27 15:27:47</t>
+          <t>2026-10-28 05:12:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2145,15 +2147,13 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G20" s="27" t="n">
-        <v>311</v>
-      </c>
+        <v>13681</v>
+      </c>
+      <c r="G20" s="27" t="n"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>app</t>
@@ -2163,17 +2163,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-27 14:45:13</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2183,13 +2183,15 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>4640</v>
-      </c>
-      <c r="G21" s="27" t="n"/>
+        <v>1401</v>
+      </c>
+      <c r="G21" s="27" t="n">
+        <v>311</v>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>app</t>
@@ -2199,7 +2201,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:39</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2219,11 +2221,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>307</v>
+        <v>4640</v>
       </c>
       <c r="G22" s="27" t="n"/>
       <c r="H22" t="inlineStr">
@@ -2235,7 +2237,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:05</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2255,11 +2257,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F23" s="27" t="n">
-        <v>3787</v>
+        <v>307</v>
       </c>
       <c r="G23" s="27" t="n"/>
       <c r="H23" t="inlineStr">
@@ -2271,7 +2273,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-27 14:41:31</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2291,11 +2293,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>4947</v>
+        <v>3787</v>
       </c>
       <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
@@ -2307,17 +2309,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2327,11 +2329,11 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>311</v>
+        <v>4947</v>
       </c>
       <c r="G25" s="27" t="n"/>
       <c r="H25" t="inlineStr">
@@ -2343,7 +2345,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2363,15 +2365,13 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G26" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G26" s="27" t="n"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>app</t>
@@ -2381,7 +2381,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2396,16 +2396,30 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n"/>
-      <c r="G27" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n">
+        <v>15809</v>
+      </c>
+      <c r="G27" s="27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2420,40 +2434,26 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n">
-        <v>1157</v>
-      </c>
-      <c r="G28" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2467,29 +2467,31 @@
         </is>
       </c>
       <c r="F29" s="27" t="n">
-        <v>8300</v>
-      </c>
-      <c r="G29" s="27" t="n"/>
+        <v>1157</v>
+      </c>
+      <c r="G29" s="27" t="n">
+        <v>911</v>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2503,21 +2505,19 @@
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G30" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>8300</v>
+      </c>
+      <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2541,9 +2541,11 @@
         </is>
       </c>
       <c r="F31" s="27" t="n">
+        <v>911</v>
+      </c>
+      <c r="G31" s="27" t="n">
         <v>351</v>
       </c>
-      <c r="G31" s="27" t="n"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>app</t>
@@ -2553,7 +2555,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2573,15 +2575,13 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G32" s="27" t="n">
-        <v>3510</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G32" s="27" t="n"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>app</t>
@@ -2591,7 +2591,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2615,10 +2615,10 @@
         </is>
       </c>
       <c r="F33" s="27" t="n">
+        <v>20274</v>
+      </c>
+      <c r="G33" s="27" t="n">
         <v>3510</v>
-      </c>
-      <c r="G33" s="27" t="n">
-        <v>351</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2629,17 +2629,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2653,29 +2653,31 @@
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>13001</v>
-      </c>
-      <c r="G34" s="27" t="n"/>
+        <v>3510</v>
+      </c>
+      <c r="G34" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2689,19 +2691,19 @@
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>351</v>
+        <v>13001</v>
       </c>
       <c r="G35" s="27" t="n"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2716,16 +2718,28 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F36" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="G36" s="27" t="n"/>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2740,40 +2754,26 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G37" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="27" t="n"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2787,29 +2787,31 @@
         </is>
       </c>
       <c r="F38" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G38" s="27" t="n"/>
+        <v>8060</v>
+      </c>
+      <c r="G38" s="27" t="n">
+        <v>122</v>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2823,21 +2825,19 @@
         </is>
       </c>
       <c r="F39" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G39" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G39" s="27" t="n"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2861,10 +2861,10 @@
         </is>
       </c>
       <c r="F40" s="27" t="n">
+        <v>122</v>
+      </c>
+      <c r="G40" s="27" t="n">
         <v>121</v>
-      </c>
-      <c r="G40" s="27" t="n">
-        <v>120</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2899,9 +2899,11 @@
         </is>
       </c>
       <c r="F41" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G41" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="G41" s="27" t="n"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>app</t>
@@ -2911,7 +2913,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2931,15 +2933,13 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F42" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G42" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G42" s="27" t="n"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>app</t>
@@ -2949,7 +2949,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2964,16 +2964,30 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n"/>
-      <c r="G43" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G43" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2988,40 +3002,26 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F44" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G44" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F44" s="27" t="n"/>
+      <c r="G44" s="27" t="n"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3031,13 +3031,15 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F45" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G45" s="27" t="n"/>
+        <v>2680</v>
+      </c>
+      <c r="G45" s="27" t="n">
+        <v>2650</v>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>app</t>
@@ -3047,7 +3049,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3067,15 +3069,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F46" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G46" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G46" s="27" t="n"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>app</t>
@@ -3085,7 +3085,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3105,11 +3105,11 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F47" s="27" t="n">
-        <v>4189</v>
+        <v>7567</v>
       </c>
       <c r="G47" s="27" t="n">
         <v>0</v>
@@ -3123,7 +3123,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3143,35 +3143,35 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F48" s="27" t="n">
-        <v>3685</v>
+        <v>4189</v>
       </c>
       <c r="G48" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3185,31 +3185,31 @@
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>2650</v>
+        <v>3685</v>
       </c>
       <c r="G49" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3223,29 +3223,31 @@
         </is>
       </c>
       <c r="F50" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G50" s="27" t="n"/>
+        <v>2650</v>
+      </c>
+      <c r="G50" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3259,21 +3261,19 @@
         </is>
       </c>
       <c r="F51" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G51" s="27" t="n">
-        <v>387</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G51" s="27" t="n"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3288,16 +3288,30 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F52" s="27" t="n"/>
-      <c r="G52" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F52" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G52" s="27" t="n">
+        <v>387</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3312,28 +3326,16 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F53" s="27" t="n">
-        <v>387</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F53" s="27" t="n"/>
       <c r="G53" s="27" t="n"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3353,15 +3355,13 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F54" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G54" s="27" t="n">
-        <v>1100</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="G54" s="27" t="n"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>app</t>
@@ -3371,17 +3371,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3395,9 +3395,11 @@
         </is>
       </c>
       <c r="F55" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G55" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G55" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>app</t>
@@ -3407,31 +3409,43 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G56" s="27" t="n"/>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3446,7 +3460,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F57" s="27" t="n"/>
@@ -3455,53 +3469,41 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F58" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F58" s="27" t="n"/>
       <c r="G58" s="27" t="n"/>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3511,47 +3513,59 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F59" s="27" t="n">
-        <v>0</v>
+        <v>10808</v>
       </c>
       <c r="G59" s="27" t="n"/>
       <c r="H59" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F60" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F60" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G60" s="27" t="n"/>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3566,7 +3580,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F61" s="27" t="n"/>
@@ -3575,22 +3589,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F62" s="27" t="n"/>
@@ -3599,7 +3613,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3614,28 +3628,16 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F63" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="n"/>
       <c r="G63" s="27" t="n"/>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3655,15 +3657,13 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F64" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G64" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G64" s="27" t="n"/>
       <c r="H64" t="inlineStr">
         <is>
           <t>app</t>
@@ -3673,7 +3673,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3688,16 +3688,30 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F65" s="27" t="n"/>
-      <c r="G65" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F65" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G65" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3712,7 +3726,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F66" s="27" t="n"/>
@@ -3721,103 +3735,91 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F67" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F67" s="27" t="n"/>
       <c r="G67" s="27" t="n"/>
-      <c r="H67" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F68" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F68" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G68" s="27" t="n"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F69" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F69" s="27" t="n"/>
       <c r="G69" s="27" t="n"/>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3832,31 +3834,43 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F70" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F70" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G70" s="27" t="n"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F71" s="27" t="n"/>
@@ -3865,7 +3879,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3880,28 +3894,16 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F72" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F72" s="27" t="n"/>
       <c r="G72" s="27" t="n"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3916,52 +3918,52 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F73" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G73" s="27" t="n"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F74" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F74" s="27" t="n"/>
       <c r="G74" s="27" t="n"/>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3976,16 +3978,28 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F75" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F75" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G75" s="27" t="n"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4000,7 +4014,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F76" s="27" t="n"/>
@@ -4009,69 +4023,69 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F77" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G77" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F77" s="27" t="n"/>
+      <c r="G77" s="27" t="n"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F78" s="27" t="n"/>
-      <c r="G78" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F78" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G78" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4086,7 +4100,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F79" s="27" t="n"/>
@@ -4095,43 +4109,31 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F80" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F80" s="27" t="n"/>
       <c r="G80" s="27" t="n"/>
-      <c r="H80" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4146,16 +4148,28 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F81" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F81" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G81" s="27" t="n"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4170,7 +4184,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F82" s="27" t="n"/>
@@ -4179,43 +4193,31 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F83" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F83" s="27" t="n"/>
       <c r="G83" s="27" t="n"/>
-      <c r="H83" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4235,11 +4237,11 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F84" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G84" s="27" t="n"/>
       <c r="H84" t="inlineStr">
@@ -4251,31 +4253,43 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F85" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F85" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G85" s="27" t="n"/>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4290,7 +4304,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
@@ -4299,7 +4313,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4314,7 +4328,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F87" s="27" t="n"/>
@@ -4323,43 +4337,31 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F88" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="n"/>
       <c r="G88" s="27" t="n"/>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4374,26 +4376,38 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F89" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G89" s="27" t="n"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4407,7 +4421,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4422,7 +4436,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F91" s="27" t="n"/>
@@ -4431,7 +4445,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4446,7 +4460,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F92" s="27" t="n"/>
@@ -4455,7 +4469,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4470,7 +4484,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F93" s="27" t="n"/>
@@ -4479,7 +4493,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4494,7 +4508,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F94" s="27" t="n"/>
@@ -4503,7 +4517,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4518,7 +4532,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F95" s="27" t="n"/>
@@ -4527,22 +4541,22 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F96" s="27" t="n"/>
@@ -4551,7 +4565,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4575,7 +4589,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4590,7 +4604,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F98" s="27" t="n"/>
@@ -4599,7 +4613,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4614,7 +4628,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F99" s="27" t="n"/>
@@ -4623,7 +4637,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4638,7 +4652,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F100" s="27" t="n"/>
@@ -4647,7 +4661,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4662,7 +4676,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F101" s="27" t="n"/>
@@ -4671,7 +4685,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4695,7 +4709,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4710,7 +4724,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F103" s="27" t="n"/>
@@ -4719,7 +4733,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4734,11 +4748,35 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F104" s="27" t="n"/>
       <c r="G104" s="27" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F105" s="27" t="n"/>
+      <c r="G105" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 2 step updates (helbert)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-30 03:28 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-30 17:14 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1160,8 +1160,12 @@
         <f>SUM(E9:AE9)</f>
         <v/>
       </c>
-      <c r="E9" s="22" t="n"/>
-      <c r="F9" s="22" t="n"/>
+      <c r="E9" s="22" t="n">
+        <v>10040</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>6257</v>
+      </c>
       <c r="G9" s="22" t="n"/>
       <c r="H9" s="22" t="n"/>
       <c r="I9" s="22" t="n"/>
@@ -1449,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H109"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1507,17 +1511,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-30 03:19:20</t>
+          <t>2026-10-30 17:14:02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1527,11 +1531,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>251</v>
+        <v>6257</v>
       </c>
       <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
@@ -1543,17 +1547,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-30 03:18:50</t>
+          <t>2026-10-30 17:13:12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1563,15 +1567,13 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>10401</v>
-      </c>
-      <c r="G3" s="27" t="n">
-        <v>2210</v>
-      </c>
+        <v>10040</v>
+      </c>
+      <c r="G3" s="27" t="n"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>app</t>
@@ -1581,17 +1583,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-30 00:00:15</t>
+          <t>2026-10-30 03:19:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1601,25 +1603,23 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>6655</v>
-      </c>
-      <c r="G4" s="27" t="n">
-        <v>30</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-29 16:26:29</t>
+          <t>2026-10-30 03:18:50</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1643,10 +1643,10 @@
         </is>
       </c>
       <c r="F5" s="27" t="n">
+        <v>10401</v>
+      </c>
+      <c r="G5" s="27" t="n">
         <v>2210</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>1011</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1657,17 +1657,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-29 14:50:59</t>
+          <t>2026-10-30 00:00:15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1677,23 +1677,25 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>10100</v>
-      </c>
-      <c r="G6" s="27" t="n"/>
+        <v>6655</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>30</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-29 14:44:19</t>
+          <t>2026-10-29 16:26:29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1717,10 +1719,10 @@
         </is>
       </c>
       <c r="F7" s="27" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G7" s="27" t="n">
         <v>1011</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>266</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1731,17 +1733,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-29 09:14:12</t>
+          <t>2026-10-29 14:50:59</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1751,23 +1753,23 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>30</v>
+        <v>10100</v>
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-29 06:32:56</t>
+          <t>2026-10-29 14:44:19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1791,9 +1793,11 @@
         </is>
       </c>
       <c r="F9" s="27" t="n">
+        <v>1011</v>
+      </c>
+      <c r="G9" s="27" t="n">
         <v>266</v>
       </c>
-      <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>app</t>
@@ -1803,17 +1807,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-29 02:35:57</t>
+          <t>2026-10-29 09:14:12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1823,35 +1827,33 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>21456</v>
-      </c>
-      <c r="G10" s="27" t="n">
-        <v>2371</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="G10" s="27" t="n"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-29 00:00:12</t>
+          <t>2026-10-29 06:32:56</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1861,23 +1863,23 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>4018</v>
+        <v>266</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-28 23:47:44</t>
+          <t>2026-10-29 02:35:57</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1901,10 +1903,10 @@
         </is>
       </c>
       <c r="F12" s="27" t="n">
+        <v>21456</v>
+      </c>
+      <c r="G12" s="27" t="n">
         <v>2371</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>371</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1915,31 +1917,43 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-28 23:46:44</t>
+          <t>2026-10-29 00:00:12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="n">
+        <v>4018</v>
+      </c>
       <c r="G13" s="27" t="n"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-28 21:24:32</t>
+          <t>2026-10-28 23:47:44</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1954,16 +1968,30 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>2371</v>
+      </c>
+      <c r="G14" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-28 17:45:48</t>
+          <t>2026-10-28 23:46:44</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1978,30 +2006,16 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>371</v>
-      </c>
-      <c r="G15" s="27" t="n">
-        <v>271</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n"/>
+      <c r="G15" s="27" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-28 10:22:51</t>
+          <t>2026-10-28 21:24:32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2016,7 +2030,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F16" s="27" t="n"/>
@@ -2025,7 +2039,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-28 06:27:01</t>
+          <t>2026-10-28 17:45:48</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2049,9 +2063,11 @@
         </is>
       </c>
       <c r="F17" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="G17" s="27" t="n">
         <v>271</v>
       </c>
-      <c r="G17" s="27" t="n"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>app</t>
@@ -2061,7 +2077,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-28 06:26:50</t>
+          <t>2026-10-28 10:22:51</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2076,40 +2092,26 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>9670</v>
-      </c>
-      <c r="G18" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n"/>
+      <c r="G18" s="27" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-28 05:23:00</t>
+          <t>2026-10-28 06:27:01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2119,11 +2121,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>10320</v>
+        <v>271</v>
       </c>
       <c r="G19" s="27" t="n"/>
       <c r="H19" t="inlineStr">
@@ -2135,17 +2137,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-28 05:21:45</t>
+          <t>2026-10-28 06:26:50</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2159,9 +2161,11 @@
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>12221</v>
-      </c>
-      <c r="G20" s="27" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>1401</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>app</t>
@@ -2171,7 +2175,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-28 05:20:41</t>
+          <t>2026-10-28 05:23:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2191,11 +2195,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>10300</v>
+        <v>10320</v>
       </c>
       <c r="G21" s="27" t="n"/>
       <c r="H21" t="inlineStr">
@@ -2207,7 +2211,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-28 05:15:21</t>
+          <t>2026-10-28 05:21:45</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2227,11 +2231,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>10595</v>
+        <v>12221</v>
       </c>
       <c r="G22" s="27" t="n"/>
       <c r="H22" t="inlineStr">
@@ -2243,7 +2247,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-28 05:13:25</t>
+          <t>2026-10-28 05:20:41</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2263,11 +2267,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F23" s="27" t="n">
-        <v>11109</v>
+        <v>10300</v>
       </c>
       <c r="G23" s="27" t="n"/>
       <c r="H23" t="inlineStr">
@@ -2279,7 +2283,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-28 05:12:16</t>
+          <t>2026-10-28 05:15:21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2299,11 +2303,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>13681</v>
+        <v>10595</v>
       </c>
       <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
@@ -2315,17 +2319,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-27 15:27:47</t>
+          <t>2026-10-28 05:13:25</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2335,15 +2339,13 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G25" s="27" t="n">
-        <v>311</v>
-      </c>
+        <v>11109</v>
+      </c>
+      <c r="G25" s="27" t="n"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>app</t>
@@ -2353,17 +2355,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-27 14:45:13</t>
+          <t>2026-10-28 05:12:16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2373,11 +2375,11 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>4640</v>
+        <v>13681</v>
       </c>
       <c r="G26" s="27" t="n"/>
       <c r="H26" t="inlineStr">
@@ -2389,17 +2391,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:39</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2409,13 +2411,15 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>307</v>
-      </c>
-      <c r="G27" s="27" t="n"/>
+        <v>1401</v>
+      </c>
+      <c r="G27" s="27" t="n">
+        <v>311</v>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
           <t>app</t>
@@ -2425,7 +2429,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:05</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2445,11 +2449,11 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F28" s="27" t="n">
-        <v>3787</v>
+        <v>4640</v>
       </c>
       <c r="G28" s="27" t="n"/>
       <c r="H28" t="inlineStr">
@@ -2461,7 +2465,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-27 14:41:31</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2481,11 +2485,11 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F29" s="27" t="n">
-        <v>4947</v>
+        <v>307</v>
       </c>
       <c r="G29" s="27" t="n"/>
       <c r="H29" t="inlineStr">
@@ -2497,17 +2501,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2517,11 +2521,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>311</v>
+        <v>3787</v>
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
@@ -2533,17 +2537,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2553,15 +2557,13 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F31" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G31" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>4947</v>
+      </c>
+      <c r="G31" s="27" t="n"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>app</t>
@@ -2571,7 +2573,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2586,16 +2588,28 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="n">
+        <v>311</v>
+      </c>
       <c r="G32" s="27" t="n"/>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2619,10 +2633,10 @@
         </is>
       </c>
       <c r="F33" s="27" t="n">
+        <v>15809</v>
+      </c>
+      <c r="G33" s="27" t="n">
         <v>1157</v>
-      </c>
-      <c r="G33" s="27" t="n">
-        <v>911</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2633,43 +2647,31 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n">
-        <v>8300</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n"/>
       <c r="G34" s="27" t="n"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2693,10 +2695,10 @@
         </is>
       </c>
       <c r="F35" s="27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="G35" s="27" t="n">
         <v>911</v>
-      </c>
-      <c r="G35" s="27" t="n">
-        <v>351</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2707,17 +2709,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2731,19 +2733,19 @@
         </is>
       </c>
       <c r="F36" s="27" t="n">
-        <v>351</v>
+        <v>8300</v>
       </c>
       <c r="G36" s="27" t="n"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2763,14 +2765,14 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F37" s="27" t="n">
-        <v>20274</v>
+        <v>911</v>
       </c>
       <c r="G37" s="27" t="n">
-        <v>3510</v>
+        <v>351</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2781,7 +2783,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2801,15 +2803,13 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F38" s="27" t="n">
-        <v>3510</v>
-      </c>
-      <c r="G38" s="27" t="n">
         <v>351</v>
       </c>
+      <c r="G38" s="27" t="n"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>app</t>
@@ -2819,17 +2819,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2843,19 +2843,21 @@
         </is>
       </c>
       <c r="F39" s="27" t="n">
-        <v>13001</v>
-      </c>
-      <c r="G39" s="27" t="n"/>
+        <v>20274</v>
+      </c>
+      <c r="G39" s="27" t="n">
+        <v>3510</v>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2879,9 +2881,11 @@
         </is>
       </c>
       <c r="F40" s="27" t="n">
+        <v>3510</v>
+      </c>
+      <c r="G40" s="27" t="n">
         <v>351</v>
       </c>
-      <c r="G40" s="27" t="n"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>app</t>
@@ -2891,31 +2895,43 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F41" s="27" t="n">
+        <v>13001</v>
+      </c>
       <c r="G41" s="27" t="n"/>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2935,15 +2951,13 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F42" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G42" s="27" t="n">
-        <v>122</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G42" s="27" t="n"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>app</t>
@@ -2953,43 +2967,31 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n">
-        <v>7493</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n"/>
       <c r="G43" s="27" t="n"/>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3013,10 +3015,10 @@
         </is>
       </c>
       <c r="F44" s="27" t="n">
+        <v>8060</v>
+      </c>
+      <c r="G44" s="27" t="n">
         <v>122</v>
-      </c>
-      <c r="G44" s="27" t="n">
-        <v>121</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -3027,17 +3029,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3051,21 +3053,19 @@
         </is>
       </c>
       <c r="F45" s="27" t="n">
-        <v>121</v>
-      </c>
-      <c r="G45" s="27" t="n">
-        <v>120</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G45" s="27" t="n"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3089,9 +3089,11 @@
         </is>
       </c>
       <c r="F46" s="27" t="n">
-        <v>120</v>
-      </c>
-      <c r="G46" s="27" t="n"/>
+        <v>122</v>
+      </c>
+      <c r="G46" s="27" t="n">
+        <v>121</v>
+      </c>
       <c r="H46" t="inlineStr">
         <is>
           <t>app</t>
@@ -3101,7 +3103,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3121,14 +3123,14 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F47" s="27" t="n">
-        <v>8981</v>
+        <v>121</v>
       </c>
       <c r="G47" s="27" t="n">
-        <v>2680</v>
+        <v>120</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3139,7 +3141,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3154,16 +3156,28 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F48" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F48" s="27" t="n">
+        <v>120</v>
+      </c>
       <c r="G48" s="27" t="n"/>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3187,10 +3201,10 @@
         </is>
       </c>
       <c r="F49" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G49" s="27" t="n">
         <v>2680</v>
-      </c>
-      <c r="G49" s="27" t="n">
-        <v>2650</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -3201,53 +3215,41 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F50" s="27" t="n">
-        <v>4933</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F50" s="27" t="n"/>
       <c r="G50" s="27" t="n"/>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3257,14 +3259,14 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F51" s="27" t="n">
-        <v>7567</v>
+        <v>2680</v>
       </c>
       <c r="G51" s="27" t="n">
-        <v>0</v>
+        <v>2650</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -3275,7 +3277,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3295,15 +3297,13 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F52" s="27" t="n">
-        <v>4189</v>
-      </c>
-      <c r="G52" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G52" s="27" t="n"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>app</t>
@@ -3313,7 +3313,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3333,35 +3333,35 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F53" s="27" t="n">
-        <v>3685</v>
+        <v>7567</v>
       </c>
       <c r="G53" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3371,14 +3371,14 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F54" s="27" t="n">
-        <v>2650</v>
+        <v>4189</v>
       </c>
       <c r="G54" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3389,7 +3389,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3413,9 +3413,11 @@
         </is>
       </c>
       <c r="F55" s="27" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G55" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="G55" s="27" t="n"/>
       <c r="H55" t="inlineStr">
         <is>
           <t>shortcut</t>
@@ -3425,7 +3427,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3449,10 +3451,10 @@
         </is>
       </c>
       <c r="F56" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G56" s="27" t="n">
         <v>831</v>
-      </c>
-      <c r="G56" s="27" t="n">
-        <v>387</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -3463,31 +3465,43 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F57" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F57" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G57" s="27" t="n"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3511,9 +3525,11 @@
         </is>
       </c>
       <c r="F58" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G58" s="27" t="n">
         <v>387</v>
       </c>
-      <c r="G58" s="27" t="n"/>
       <c r="H58" t="inlineStr">
         <is>
           <t>app</t>
@@ -3523,7 +3539,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3538,40 +3554,26 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G59" s="27" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n"/>
+      <c r="G59" s="27" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3581,11 +3583,11 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F60" s="27" t="n">
-        <v>9097</v>
+        <v>387</v>
       </c>
       <c r="G60" s="27" t="n"/>
       <c r="H60" t="inlineStr">
@@ -3597,190 +3599,216 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F61" s="27" t="n"/>
-      <c r="G61" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F61" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G61" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F62" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F62" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G62" s="27" t="n"/>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F63" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="n"/>
       <c r="G63" s="27" t="n"/>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F64" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F64" s="27" t="n"/>
       <c r="G64" s="27" t="n"/>
-      <c r="H64" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F65" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F65" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G65" s="27" t="n"/>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F66" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F66" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G66" s="27" t="n"/>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F67" s="27" t="n"/>
@@ -3789,43 +3817,31 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F68" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F68" s="27" t="n"/>
       <c r="G68" s="27" t="n"/>
-      <c r="H68" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3840,30 +3856,16 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F69" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G69" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H69" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F69" s="27" t="n"/>
+      <c r="G69" s="27" t="n"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3878,16 +3880,28 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F70" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F70" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G70" s="27" t="n"/>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3902,52 +3916,54 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F71" s="27" t="n"/>
-      <c r="G71" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F71" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G71" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F72" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F72" s="27" t="n"/>
       <c r="G72" s="27" t="n"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3962,7 +3978,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>unstory</t>
         </is>
       </c>
       <c r="F73" s="27" t="n"/>
@@ -3971,17 +3987,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3995,34 +4011,34 @@
         </is>
       </c>
       <c r="F74" s="27" t="n">
-        <v>0</v>
+        <v>4842</v>
       </c>
       <c r="G74" s="27" t="n"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F75" s="27" t="n"/>
@@ -4031,67 +4047,67 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F76" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F76" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G76" s="27" t="n"/>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F77" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F77" s="27" t="n"/>
       <c r="G77" s="27" t="n"/>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4106,7 +4122,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F78" s="27" t="n"/>
@@ -4115,17 +4131,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4139,7 +4155,7 @@
         </is>
       </c>
       <c r="F79" s="27" t="n">
-        <v>5345</v>
+        <v>12641</v>
       </c>
       <c r="G79" s="27" t="n"/>
       <c r="H79" t="inlineStr">
@@ -4151,22 +4167,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -4175,7 +4191,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4190,69 +4206,67 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F81" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F81" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G81" s="27" t="n"/>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F82" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G82" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F82" s="27" t="n"/>
+      <c r="G82" s="27" t="n"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F83" s="27" t="n"/>
@@ -4261,82 +4275,84 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F84" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G84" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F85" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F85" s="27" t="n"/>
       <c r="G85" s="27" t="n"/>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
@@ -4345,7 +4361,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4360,136 +4376,148 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F87" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F87" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G87" s="27" t="n"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F88" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="n"/>
       <c r="G88" s="27" t="n"/>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F89" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="n"/>
       <c r="G89" s="27" t="n"/>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F90" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G90" s="27" t="n"/>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F91" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F91" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G91" s="27" t="n"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4504,7 +4532,7 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F92" s="27" t="n"/>
@@ -4513,53 +4541,41 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F93" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F93" s="27" t="n"/>
       <c r="G93" s="27" t="n"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4573,46 +4589,58 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F95" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F95" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G95" s="27" t="n"/>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F96" s="27" t="n"/>
@@ -4621,7 +4649,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4645,7 +4673,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4669,7 +4697,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4684,7 +4712,7 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F99" s="27" t="n"/>
@@ -4693,7 +4721,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4708,7 +4736,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F100" s="27" t="n"/>
@@ -4717,22 +4745,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F101" s="27" t="n"/>
@@ -4741,22 +4769,22 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F102" s="27" t="n"/>
@@ -4765,7 +4793,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4780,7 +4808,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F103" s="27" t="n"/>
@@ -4789,7 +4817,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4813,7 +4841,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4837,7 +4865,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -4861,7 +4889,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -4876,7 +4904,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F107" s="27" t="n"/>
@@ -4885,7 +4913,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -4900,7 +4928,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F108" s="27" t="n"/>
@@ -4909,7 +4937,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -4924,11 +4952,59 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F109" s="27" t="n"/>
       <c r="G109" s="27" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F110" s="27" t="n"/>
+      <c r="G110" s="27" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F111" s="27" t="n"/>
+      <c r="G111" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 8 step updates (helbert)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-30 17:14 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-30 17:21 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1166,14 +1166,30 @@
       <c r="F9" s="22" t="n">
         <v>6257</v>
       </c>
-      <c r="G9" s="22" t="n"/>
-      <c r="H9" s="22" t="n"/>
-      <c r="I9" s="22" t="n"/>
-      <c r="J9" s="22" t="n"/>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="23" t="n"/>
-      <c r="M9" s="23" t="n"/>
-      <c r="N9" s="23" t="n"/>
+      <c r="G9" s="22" t="n">
+        <v>12079</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>9406</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>7034</v>
+      </c>
+      <c r="J9" s="22" t="n">
+        <v>17611</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>11079</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>7349</v>
+      </c>
+      <c r="M9" s="23" t="n">
+        <v>3691</v>
+      </c>
+      <c r="N9" s="23" t="n">
+        <v>6694</v>
+      </c>
       <c r="O9" s="23" t="n"/>
       <c r="P9" s="23" t="n"/>
       <c r="Q9" s="23" t="n"/>
@@ -1453,7 +1469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1511,7 +1527,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-30 17:14:02</t>
+          <t>2026-10-30 17:19:03</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1531,11 +1547,11 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F2" s="27" t="n">
-        <v>6257</v>
+        <v>6694</v>
       </c>
       <c r="G2" s="27" t="n"/>
       <c r="H2" t="inlineStr">
@@ -1547,7 +1563,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-30 17:13:12</t>
+          <t>2026-10-30 17:18:03</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1567,11 +1583,11 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>10040</v>
+        <v>3691</v>
       </c>
       <c r="G3" s="27" t="n"/>
       <c r="H3" t="inlineStr">
@@ -1583,17 +1599,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-30 03:19:20</t>
+          <t>2026-10-30 17:17:24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1603,11 +1619,11 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F4" s="27" t="n">
-        <v>251</v>
+        <v>7349</v>
       </c>
       <c r="G4" s="27" t="n"/>
       <c r="H4" t="inlineStr">
@@ -1619,17 +1635,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-30 03:18:50</t>
+          <t>2026-10-30 17:16:48</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1639,15 +1655,13 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F5" s="27" t="n">
-        <v>10401</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>2210</v>
-      </c>
+        <v>11079</v>
+      </c>
+      <c r="G5" s="27" t="n"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>app</t>
@@ -1657,17 +1671,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-30 00:00:15</t>
+          <t>2026-10-30 17:16:22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1677,35 +1691,33 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>6655</v>
-      </c>
-      <c r="G6" s="27" t="n">
-        <v>30</v>
-      </c>
+        <v>17611</v>
+      </c>
+      <c r="G6" s="27" t="n"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-29 16:26:29</t>
+          <t>2026-10-30 17:15:49</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1715,15 +1727,13 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>2210</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>1011</v>
-      </c>
+        <v>7034</v>
+      </c>
+      <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>app</t>
@@ -1733,17 +1743,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-29 14:50:59</t>
+          <t>2026-10-30 17:15:14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1753,11 +1763,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>10100</v>
+        <v>9406</v>
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
@@ -1769,17 +1779,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-29 14:44:19</t>
+          <t>2026-10-30 17:14:44</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1789,15 +1799,13 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>1011</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>266</v>
-      </c>
+        <v>12079</v>
+      </c>
+      <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>app</t>
@@ -1807,17 +1815,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-29 09:14:12</t>
+          <t>2026-10-30 17:14:02</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1827,33 +1835,33 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>30</v>
+        <v>6257</v>
       </c>
       <c r="G10" s="27" t="n"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-29 06:32:56</t>
+          <t>2026-10-30 17:13:12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1863,11 +1871,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>266</v>
+        <v>10040</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
@@ -1879,7 +1887,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-29 02:35:57</t>
+          <t>2026-10-30 03:19:20</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1899,15 +1907,13 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>21456</v>
-      </c>
-      <c r="G12" s="27" t="n">
-        <v>2371</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>app</t>
@@ -1917,17 +1923,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-29 00:00:12</t>
+          <t>2026-10-30 03:18:50</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1937,33 +1943,35 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>4018</v>
-      </c>
-      <c r="G13" s="27" t="n"/>
+        <v>10401</v>
+      </c>
+      <c r="G13" s="27" t="n">
+        <v>2210</v>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-28 23:47:44</t>
+          <t>2026-10-30 00:00:15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1973,25 +1981,25 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>2371</v>
+        <v>6655</v>
       </c>
       <c r="G14" s="27" t="n">
-        <v>371</v>
+        <v>30</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-28 23:46:44</t>
+          <t>2026-10-29 16:26:29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2006,40 +2014,66 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G15" s="27" t="n">
+        <v>1011</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-28 21:24:32</t>
+          <t>2026-10-29 14:50:59</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="n">
+        <v>10100</v>
+      </c>
       <c r="G16" s="27" t="n"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-28 17:45:48</t>
+          <t>2026-10-29 14:44:19</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2059,14 +2093,14 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>371</v>
+        <v>1011</v>
       </c>
       <c r="G17" s="27" t="n">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -2077,31 +2111,43 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-28 10:22:51</t>
+          <t>2026-10-29 09:14:12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="n">
+        <v>30</v>
+      </c>
       <c r="G18" s="27" t="n"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-28 06:27:01</t>
+          <t>2026-10-29 06:32:56</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2121,11 +2167,11 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="G19" s="27" t="n"/>
       <c r="H19" t="inlineStr">
@@ -2137,7 +2183,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-28 06:26:50</t>
+          <t>2026-10-29 02:35:57</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2157,14 +2203,14 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>9670</v>
+        <v>21456</v>
       </c>
       <c r="G20" s="27" t="n">
-        <v>1401</v>
+        <v>2371</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2175,17 +2221,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-28 05:23:00</t>
+          <t>2026-10-29 00:00:12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2195,33 +2241,33 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>10320</v>
+        <v>4018</v>
       </c>
       <c r="G21" s="27" t="n"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-28 05:21:45</t>
+          <t>2026-10-28 23:47:44</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2231,13 +2277,15 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>12221</v>
-      </c>
-      <c r="G22" s="27" t="n"/>
+        <v>2371</v>
+      </c>
+      <c r="G22" s="27" t="n">
+        <v>371</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>app</t>
@@ -2247,89 +2295,65 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-28 05:20:41</t>
+          <t>2026-10-28 23:46:44</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>10300</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="n"/>
       <c r="G23" s="27" t="n"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-28 05:15:21</t>
+          <t>2026-10-28 21:24:32</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n">
-        <v>10595</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="n"/>
       <c r="G24" s="27" t="n"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-28 05:13:25</t>
+          <t>2026-10-28 17:45:48</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2339,13 +2363,15 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>11109</v>
-      </c>
-      <c r="G25" s="27" t="n"/>
+        <v>371</v>
+      </c>
+      <c r="G25" s="27" t="n">
+        <v>271</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>app</t>
@@ -2355,43 +2381,31 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-28 05:12:16</t>
+          <t>2026-10-28 10:22:51</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n">
-        <v>13681</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="n"/>
       <c r="G26" s="27" t="n"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-27 15:27:47</t>
+          <t>2026-10-28 06:27:01</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2411,15 +2425,13 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F27" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G27" s="27" t="n">
-        <v>311</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="G27" s="27" t="n"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>app</t>
@@ -2429,17 +2441,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-27 14:45:13</t>
+          <t>2026-10-28 06:26:50</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2449,13 +2461,15 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F28" s="27" t="n">
-        <v>4640</v>
-      </c>
-      <c r="G28" s="27" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="G28" s="27" t="n">
+        <v>1401</v>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>app</t>
@@ -2465,17 +2479,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:39</t>
+          <t>2026-10-28 05:23:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2489,7 +2503,7 @@
         </is>
       </c>
       <c r="F29" s="27" t="n">
-        <v>307</v>
+        <v>10320</v>
       </c>
       <c r="G29" s="27" t="n"/>
       <c r="H29" t="inlineStr">
@@ -2501,17 +2515,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:05</t>
+          <t>2026-10-28 05:21:45</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2521,11 +2535,11 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F30" s="27" t="n">
-        <v>3787</v>
+        <v>12221</v>
       </c>
       <c r="G30" s="27" t="n"/>
       <c r="H30" t="inlineStr">
@@ -2537,17 +2551,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-27 14:41:31</t>
+          <t>2026-10-28 05:20:41</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2557,11 +2571,11 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F31" s="27" t="n">
-        <v>4947</v>
+        <v>10300</v>
       </c>
       <c r="G31" s="27" t="n"/>
       <c r="H31" t="inlineStr">
@@ -2573,17 +2587,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-28 05:15:21</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2593,11 +2607,11 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>311</v>
+        <v>10595</v>
       </c>
       <c r="G32" s="27" t="n"/>
       <c r="H32" t="inlineStr">
@@ -2609,17 +2623,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-28 05:13:25</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2629,15 +2643,13 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F33" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G33" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>11109</v>
+      </c>
+      <c r="G33" s="27" t="n"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>app</t>
@@ -2647,31 +2659,43 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-28 05:12:16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>13681</v>
+      </c>
       <c r="G34" s="27" t="n"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2691,14 +2715,14 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>1157</v>
+        <v>1401</v>
       </c>
       <c r="G35" s="27" t="n">
-        <v>911</v>
+        <v>311</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2709,17 +2733,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2733,29 +2757,29 @@
         </is>
       </c>
       <c r="F36" s="27" t="n">
-        <v>8300</v>
+        <v>4640</v>
       </c>
       <c r="G36" s="27" t="n"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2765,15 +2789,13 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F37" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G37" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>307</v>
+      </c>
+      <c r="G37" s="27" t="n"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>app</t>
@@ -2783,17 +2805,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2803,11 +2825,11 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F38" s="27" t="n">
-        <v>351</v>
+        <v>3787</v>
       </c>
       <c r="G38" s="27" t="n"/>
       <c r="H38" t="inlineStr">
@@ -2819,17 +2841,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2839,15 +2861,13 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F39" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G39" s="27" t="n">
-        <v>3510</v>
-      </c>
+        <v>4947</v>
+      </c>
+      <c r="G39" s="27" t="n"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>app</t>
@@ -2857,7 +2877,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2877,15 +2897,13 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
-        <v>3510</v>
-      </c>
-      <c r="G40" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G40" s="27" t="n"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>app</t>
@@ -2895,17 +2913,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2915,23 +2933,25 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F41" s="27" t="n">
-        <v>13001</v>
-      </c>
-      <c r="G41" s="27" t="n"/>
+        <v>15809</v>
+      </c>
+      <c r="G41" s="27" t="n">
+        <v>1157</v>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2946,28 +2966,16 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>2026-10-25</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n">
-        <v>351</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F42" s="27" t="n"/>
       <c r="G42" s="27" t="n"/>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2982,26 +2990,40 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n"/>
-      <c r="G43" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="F43" s="27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="G43" s="27" t="n">
+        <v>911</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3011,35 +3033,33 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F44" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G44" s="27" t="n">
-        <v>122</v>
-      </c>
+        <v>8300</v>
+      </c>
+      <c r="G44" s="27" t="n"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3049,23 +3069,25 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F45" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G45" s="27" t="n"/>
+        <v>911</v>
+      </c>
+      <c r="G45" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3085,15 +3107,13 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F46" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G46" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G46" s="27" t="n"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>app</t>
@@ -3103,7 +3123,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3123,14 +3143,14 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F47" s="27" t="n">
-        <v>121</v>
+        <v>20274</v>
       </c>
       <c r="G47" s="27" t="n">
-        <v>120</v>
+        <v>3510</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -3141,7 +3161,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3161,13 +3181,15 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F48" s="27" t="n">
-        <v>120</v>
-      </c>
-      <c r="G48" s="27" t="n"/>
+        <v>3510</v>
+      </c>
+      <c r="G48" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
           <t>app</t>
@@ -3177,17 +3199,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3197,25 +3219,23 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G49" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>13001</v>
+      </c>
+      <c r="G49" s="27" t="n"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3230,16 +3250,28 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F50" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F50" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="G50" s="27" t="n"/>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3254,40 +3286,26 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F51" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G51" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F51" s="27" t="n"/>
+      <c r="G51" s="27" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3297,13 +3315,15 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F52" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G52" s="27" t="n"/>
+        <v>8060</v>
+      </c>
+      <c r="G52" s="27" t="n">
+        <v>122</v>
+      </c>
       <c r="H52" t="inlineStr">
         <is>
           <t>app</t>
@@ -3313,7 +3333,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3333,35 +3353,33 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F53" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G53" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G53" s="27" t="n"/>
       <c r="H53" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3371,14 +3389,14 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F54" s="27" t="n">
-        <v>4189</v>
+        <v>122</v>
       </c>
       <c r="G54" s="27" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3389,17 +3407,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3409,25 +3427,25 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F55" s="27" t="n">
-        <v>3685</v>
+        <v>121</v>
       </c>
       <c r="G55" s="27" t="n">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3447,15 +3465,13 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F56" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="G56" s="27" t="n">
-        <v>831</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G56" s="27" t="n"/>
       <c r="H56" t="inlineStr">
         <is>
           <t>app</t>
@@ -3465,17 +3481,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3489,19 +3505,21 @@
         </is>
       </c>
       <c r="F57" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" s="27" t="n"/>
+        <v>8981</v>
+      </c>
+      <c r="G57" s="27" t="n">
+        <v>2680</v>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3516,30 +3534,16 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F58" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G58" s="27" t="n">
-        <v>387</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F58" s="27" t="n"/>
+      <c r="G58" s="27" t="n"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3554,26 +3558,40 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F59" s="27" t="n"/>
-      <c r="G59" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F59" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="G59" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3583,11 +3601,11 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F60" s="27" t="n">
-        <v>387</v>
+        <v>4933</v>
       </c>
       <c r="G60" s="27" t="n"/>
       <c r="H60" t="inlineStr">
@@ -3599,17 +3617,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3619,14 +3637,14 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F61" s="27" t="n">
-        <v>9720</v>
+        <v>7567</v>
       </c>
       <c r="G61" s="27" t="n">
-        <v>1100</v>
+        <v>0</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
@@ -3637,17 +3655,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3661,9 +3679,11 @@
         </is>
       </c>
       <c r="F62" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G62" s="27" t="n"/>
+        <v>4189</v>
+      </c>
+      <c r="G62" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>app</t>
@@ -3673,65 +3693,93 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F63" s="27" t="n"/>
-      <c r="G63" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="n">
+        <v>3685</v>
+      </c>
+      <c r="G63" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F64" s="27" t="n"/>
-      <c r="G64" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F64" s="27" t="n">
+        <v>2650</v>
+      </c>
+      <c r="G64" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3741,33 +3789,33 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F65" s="27" t="n">
-        <v>10808</v>
+        <v>0</v>
       </c>
       <c r="G65" s="27" t="n"/>
       <c r="H65" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3777,38 +3825,40 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F66" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G66" s="27" t="n"/>
+        <v>831</v>
+      </c>
+      <c r="G66" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>approved</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F67" s="27" t="n"/>
@@ -3817,31 +3867,43 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F68" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F68" s="27" t="n">
+        <v>387</v>
+      </c>
       <c r="G68" s="27" t="n"/>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3856,26 +3918,40 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F69" s="27" t="n"/>
-      <c r="G69" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F69" s="27" t="n">
+        <v>9720</v>
+      </c>
+      <c r="G69" s="27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3889,7 +3965,7 @@
         </is>
       </c>
       <c r="F70" s="27" t="n">
-        <v>1100</v>
+        <v>9097</v>
       </c>
       <c r="G70" s="27" t="n"/>
       <c r="H70" t="inlineStr">
@@ -3901,60 +3977,46 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F71" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G71" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="H71" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F71" s="27" t="n"/>
+      <c r="G71" s="27" t="n"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F72" s="27" t="n"/>
@@ -3963,41 +4025,53 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>unstory</t>
-        </is>
-      </c>
-      <c r="F73" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>10808</v>
+      </c>
       <c r="G73" s="27" t="n"/>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4007,38 +4081,38 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F74" s="27" t="n">
-        <v>4842</v>
+        <v>0</v>
       </c>
       <c r="G74" s="27" t="n"/>
       <c r="H74" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F75" s="27" t="n"/>
@@ -4047,58 +4121,46 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F76" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F76" s="27" t="n"/>
       <c r="G76" s="27" t="n"/>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F77" s="27" t="n"/>
@@ -4107,41 +4169,53 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F78" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F78" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="G78" s="27" t="n"/>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4151,13 +4225,15 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F79" s="27" t="n">
-        <v>12641</v>
-      </c>
-      <c r="G79" s="27" t="n"/>
+        <v>18461</v>
+      </c>
+      <c r="G79" s="27" t="n">
+        <v>1985</v>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>app</t>
@@ -4167,22 +4243,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -4191,43 +4267,31 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F81" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F81" s="27" t="n"/>
       <c r="G81" s="27" t="n"/>
-      <c r="H81" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4242,31 +4306,43 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F82" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F82" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G82" s="27" t="n"/>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F83" s="27" t="n"/>
@@ -4275,17 +4351,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4299,36 +4375,34 @@
         </is>
       </c>
       <c r="F84" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G84" s="27" t="n">
-        <v>100</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G84" s="27" t="n"/>
       <c r="H84" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F85" s="27" t="n"/>
@@ -4337,22 +4411,22 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F86" s="27" t="n"/>
@@ -4361,17 +4435,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4385,7 +4459,7 @@
         </is>
       </c>
       <c r="F87" s="27" t="n">
-        <v>10383</v>
+        <v>12641</v>
       </c>
       <c r="G87" s="27" t="n"/>
       <c r="H87" t="inlineStr">
@@ -4397,22 +4471,22 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F88" s="27" t="n"/>
@@ -4421,137 +4495,139 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F89" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G89" s="27" t="n"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F90" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="n"/>
       <c r="G90" s="27" t="n"/>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F91" s="27" t="n">
-        <v>9060</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F91" s="27" t="n"/>
       <c r="G91" s="27" t="n"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F92" s="27" t="n"/>
-      <c r="G92" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F92" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G92" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4565,17 +4641,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4589,17 +4665,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4613,7 +4689,7 @@
         </is>
       </c>
       <c r="F95" s="27" t="n">
-        <v>6310</v>
+        <v>10383</v>
       </c>
       <c r="G95" s="27" t="n"/>
       <c r="H95" t="inlineStr">
@@ -4625,22 +4701,22 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F96" s="27" t="n"/>
@@ -4649,17 +4725,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4673,70 +4749,94 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>reset</t>
-        </is>
-      </c>
-      <c r="F98" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F98" s="27" t="n">
+        <v>100</v>
+      </c>
       <c r="G98" s="27" t="n"/>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F99" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F99" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G99" s="27" t="n"/>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F100" s="27" t="n"/>
@@ -4745,22 +4845,22 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F101" s="27" t="n"/>
@@ -4769,17 +4869,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4793,46 +4893,58 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>requested</t>
-        </is>
-      </c>
-      <c r="F103" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F103" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G103" s="27" t="n"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F104" s="27" t="n"/>
@@ -4841,22 +4953,22 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F105" s="27" t="n"/>
@@ -4865,22 +4977,22 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F106" s="27" t="n"/>
@@ -4889,22 +5001,22 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F107" s="27" t="n"/>
@@ -4913,22 +5025,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F108" s="27" t="n"/>
@@ -4937,22 +5049,22 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F109" s="27" t="n"/>
@@ -4961,22 +5073,22 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F110" s="27" t="n"/>
@@ -4985,7 +5097,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5000,11 +5112,203 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F111" s="27" t="n"/>
       <c r="G111" s="27" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:41:34</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F112" s="27" t="n"/>
+      <c r="G112" s="27" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:41:28</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F113" s="27" t="n"/>
+      <c r="G113" s="27" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:27:02</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F114" s="27" t="n"/>
+      <c r="G114" s="27" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:22:11</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>denied</t>
+        </is>
+      </c>
+      <c r="F115" s="27" t="n"/>
+      <c r="G115" s="27" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-10-20 20:20:27</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F116" s="27" t="n"/>
+      <c r="G116" s="27" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:58:34</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F117" s="27" t="n"/>
+      <c r="G117" s="27" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:19</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F118" s="27" t="n"/>
+      <c r="G118" s="27" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F119" s="27" t="n"/>
+      <c r="G119" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
data: 1 account event (sidnei)
</commit_message>
<xml_diff>
--- a/step-tracking_Team8.xlsx
+++ b/step-tracking_Team8.xlsx
@@ -596,7 +596,7 @@
     <row r="1">
       <c r="B1" s="21" t="inlineStr">
         <is>
-          <t>Updated 2026-10-31 01:38 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
+          <t>Updated 2026-10-31 16:07 UTC by the Nokia - Step Challenge 2026 - Team 8 app</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1471,7 +1471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1529,55 +1529,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-31 01:37:24</t>
+          <t>2026-10-31 15:58:33</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>sidnei</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Sidnei Marcos Guerbali</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="F2" s="27" t="n">
-        <v>9861</v>
-      </c>
-      <c r="G2" s="27" t="n">
-        <v>2510</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="n"/>
+      <c r="G2" s="27" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-31 00:00:13</t>
+          <t>2026-10-31 01:37:24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1591,43 +1577,57 @@
         </is>
       </c>
       <c r="F3" s="27" t="n">
-        <v>14622</v>
-      </c>
-      <c r="G3" s="27" t="n"/>
+        <v>9861</v>
+      </c>
+      <c r="G3" s="27" t="n">
+        <v>2510</v>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-30 21:16:06</t>
+          <t>2026-10-31 00:00:13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="n">
+        <v>14622</v>
+      </c>
       <c r="G4" s="27" t="n"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-30 18:18:20</t>
+          <t>2026-10-30 21:16:06</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1642,40 +1642,26 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n">
-        <v>2510</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>251</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-30 17:19:03</t>
+          <t>2026-10-30 18:18:20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1685,13 +1671,15 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F6" s="27" t="n">
-        <v>6694</v>
-      </c>
-      <c r="G6" s="27" t="n"/>
+        <v>2510</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>251</v>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>app</t>
@@ -1701,7 +1689,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-30 17:18:03</t>
+          <t>2026-10-30 17:19:03</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1721,11 +1709,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F7" s="27" t="n">
-        <v>3691</v>
+        <v>6694</v>
       </c>
       <c r="G7" s="27" t="n"/>
       <c r="H7" t="inlineStr">
@@ -1737,7 +1725,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-30 17:17:24</t>
+          <t>2026-10-30 17:18:03</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1757,11 +1745,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F8" s="27" t="n">
-        <v>7349</v>
+        <v>3691</v>
       </c>
       <c r="G8" s="27" t="n"/>
       <c r="H8" t="inlineStr">
@@ -1773,7 +1761,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-30 17:16:48</t>
+          <t>2026-10-30 17:17:24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1793,11 +1781,11 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F9" s="27" t="n">
-        <v>11079</v>
+        <v>7349</v>
       </c>
       <c r="G9" s="27" t="n"/>
       <c r="H9" t="inlineStr">
@@ -1809,7 +1797,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-30 17:16:22</t>
+          <t>2026-10-30 17:16:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1829,11 +1817,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F10" s="27" t="n">
-        <v>17611</v>
+        <v>11079</v>
       </c>
       <c r="G10" s="27" t="n"/>
       <c r="H10" t="inlineStr">
@@ -1845,7 +1833,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-30 17:15:49</t>
+          <t>2026-10-30 17:16:22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1865,11 +1853,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F11" s="27" t="n">
-        <v>7034</v>
+        <v>17611</v>
       </c>
       <c r="G11" s="27" t="n"/>
       <c r="H11" t="inlineStr">
@@ -1881,7 +1869,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-30 17:15:14</t>
+          <t>2026-10-30 17:15:49</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1901,11 +1889,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>9406</v>
+        <v>7034</v>
       </c>
       <c r="G12" s="27" t="n"/>
       <c r="H12" t="inlineStr">
@@ -1917,7 +1905,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-30 17:14:44</t>
+          <t>2026-10-30 17:15:14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1937,11 +1925,11 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F13" s="27" t="n">
-        <v>12079</v>
+        <v>9406</v>
       </c>
       <c r="G13" s="27" t="n"/>
       <c r="H13" t="inlineStr">
@@ -1953,7 +1941,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-30 17:14:02</t>
+          <t>2026-10-30 17:14:44</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1973,11 +1961,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F14" s="27" t="n">
-        <v>6257</v>
+        <v>12079</v>
       </c>
       <c r="G14" s="27" t="n"/>
       <c r="H14" t="inlineStr">
@@ -1989,7 +1977,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-30 17:13:12</t>
+          <t>2026-10-30 17:14:02</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2009,11 +1997,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F15" s="27" t="n">
-        <v>10040</v>
+        <v>6257</v>
       </c>
       <c r="G15" s="27" t="n"/>
       <c r="H15" t="inlineStr">
@@ -2025,17 +2013,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-30 03:19:20</t>
+          <t>2026-10-30 17:13:12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2045,11 +2033,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>251</v>
+        <v>10040</v>
       </c>
       <c r="G16" s="27" t="n"/>
       <c r="H16" t="inlineStr">
@@ -2061,7 +2049,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-30 03:18:50</t>
+          <t>2026-10-30 03:19:20</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2081,15 +2069,13 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="F17" s="27" t="n">
-        <v>10401</v>
-      </c>
-      <c r="G17" s="27" t="n">
-        <v>2210</v>
-      </c>
+        <v>251</v>
+      </c>
+      <c r="G17" s="27" t="n"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>app</t>
@@ -2099,17 +2085,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-30 00:00:15</t>
+          <t>2026-10-30 03:18:50</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2123,31 +2109,31 @@
         </is>
       </c>
       <c r="F18" s="27" t="n">
-        <v>6655</v>
+        <v>10401</v>
       </c>
       <c r="G18" s="27" t="n">
-        <v>30</v>
+        <v>2210</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-29 16:26:29</t>
+          <t>2026-10-30 00:00:15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2161,31 +2147,31 @@
         </is>
       </c>
       <c r="F19" s="27" t="n">
-        <v>2210</v>
+        <v>6655</v>
       </c>
       <c r="G19" s="27" t="n">
-        <v>1011</v>
+        <v>30</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-29 14:50:59</t>
+          <t>2026-10-29 16:26:29</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2195,13 +2181,15 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F20" s="27" t="n">
-        <v>10100</v>
-      </c>
-      <c r="G20" s="27" t="n"/>
+        <v>2210</v>
+      </c>
+      <c r="G20" s="27" t="n">
+        <v>1011</v>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>app</t>
@@ -2211,17 +2199,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-29 14:44:19</t>
+          <t>2026-10-29 14:50:59</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2231,15 +2219,13 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F21" s="27" t="n">
-        <v>1011</v>
-      </c>
-      <c r="G21" s="27" t="n">
-        <v>266</v>
-      </c>
+        <v>10100</v>
+      </c>
+      <c r="G21" s="27" t="n"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>app</t>
@@ -2249,17 +2235,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-29 09:14:12</t>
+          <t>2026-10-29 14:44:19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2273,29 +2259,31 @@
         </is>
       </c>
       <c r="F22" s="27" t="n">
-        <v>30</v>
-      </c>
-      <c r="G22" s="27" t="n"/>
+        <v>1011</v>
+      </c>
+      <c r="G22" s="27" t="n">
+        <v>266</v>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-29 06:32:56</t>
+          <t>2026-10-29 09:14:12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2309,19 +2297,19 @@
         </is>
       </c>
       <c r="F23" s="27" t="n">
-        <v>266</v>
+        <v>30</v>
       </c>
       <c r="G23" s="27" t="n"/>
       <c r="H23" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-29 02:35:57</t>
+          <t>2026-10-29 06:32:56</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2341,15 +2329,13 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="F24" s="27" t="n">
-        <v>21456</v>
-      </c>
-      <c r="G24" s="27" t="n">
-        <v>2371</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="G24" s="27" t="n"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>app</t>
@@ -2359,17 +2345,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-29 00:00:12</t>
+          <t>2026-10-29 02:35:57</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2383,29 +2369,31 @@
         </is>
       </c>
       <c r="F25" s="27" t="n">
-        <v>4018</v>
-      </c>
-      <c r="G25" s="27" t="n"/>
+        <v>21456</v>
+      </c>
+      <c r="G25" s="27" t="n">
+        <v>2371</v>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-28 23:47:44</t>
+          <t>2026-10-29 00:00:12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2419,21 +2407,19 @@
         </is>
       </c>
       <c r="F26" s="27" t="n">
-        <v>2371</v>
-      </c>
-      <c r="G26" s="27" t="n">
-        <v>371</v>
-      </c>
+        <v>4018</v>
+      </c>
+      <c r="G26" s="27" t="n"/>
       <c r="H26" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-28 23:46:44</t>
+          <t>2026-10-28 23:47:44</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2448,16 +2434,30 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n"/>
-      <c r="G27" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="n">
+        <v>2371</v>
+      </c>
+      <c r="G27" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-28 21:24:32</t>
+          <t>2026-10-28 23:46:44</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2472,7 +2472,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F28" s="27" t="n"/>
@@ -2481,7 +2481,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-28 17:45:48</t>
+          <t>2026-10-28 21:24:32</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -2496,30 +2496,16 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n">
-        <v>371</v>
-      </c>
-      <c r="G29" s="27" t="n">
-        <v>271</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="n"/>
+      <c r="G29" s="27" t="n"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-28 10:22:51</t>
+          <t>2026-10-28 17:45:48</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2534,16 +2520,30 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n"/>
-      <c r="G30" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>371</v>
+      </c>
+      <c r="G30" s="27" t="n">
+        <v>271</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-28 06:27:01</t>
+          <t>2026-10-28 10:22:51</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2558,28 +2558,16 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>2026-10-28</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
-        <v>271</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="n"/>
       <c r="G31" s="27" t="n"/>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-28 06:26:50</t>
+          <t>2026-10-28 06:27:01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -2599,15 +2587,13 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="F32" s="27" t="n">
-        <v>9670</v>
-      </c>
-      <c r="G32" s="27" t="n">
-        <v>1401</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="G32" s="27" t="n"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>app</t>
@@ -2617,17 +2603,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-28 05:23:00</t>
+          <t>2026-10-28 06:26:50</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2637,13 +2623,15 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F33" s="27" t="n">
-        <v>10320</v>
-      </c>
-      <c r="G33" s="27" t="n"/>
+        <v>9670</v>
+      </c>
+      <c r="G33" s="27" t="n">
+        <v>1401</v>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
           <t>app</t>
@@ -2653,7 +2641,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-28 05:21:45</t>
+          <t>2026-10-28 05:23:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2673,11 +2661,11 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F34" s="27" t="n">
-        <v>12221</v>
+        <v>10320</v>
       </c>
       <c r="G34" s="27" t="n"/>
       <c r="H34" t="inlineStr">
@@ -2689,7 +2677,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-28 05:20:41</t>
+          <t>2026-10-28 05:21:45</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2709,11 +2697,11 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F35" s="27" t="n">
-        <v>10300</v>
+        <v>12221</v>
       </c>
       <c r="G35" s="27" t="n"/>
       <c r="H35" t="inlineStr">
@@ -2725,7 +2713,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-28 05:15:21</t>
+          <t>2026-10-28 05:20:41</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2745,11 +2733,11 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F36" s="27" t="n">
-        <v>10595</v>
+        <v>10300</v>
       </c>
       <c r="G36" s="27" t="n"/>
       <c r="H36" t="inlineStr">
@@ -2761,7 +2749,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-28 05:13:25</t>
+          <t>2026-10-28 05:15:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2781,11 +2769,11 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F37" s="27" t="n">
-        <v>11109</v>
+        <v>10595</v>
       </c>
       <c r="G37" s="27" t="n"/>
       <c r="H37" t="inlineStr">
@@ -2797,7 +2785,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-28 05:12:16</t>
+          <t>2026-10-28 05:13:25</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2817,11 +2805,11 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F38" s="27" t="n">
-        <v>13681</v>
+        <v>11109</v>
       </c>
       <c r="G38" s="27" t="n"/>
       <c r="H38" t="inlineStr">
@@ -2833,17 +2821,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-27 15:27:47</t>
+          <t>2026-10-28 05:12:16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2853,15 +2841,13 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F39" s="27" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G39" s="27" t="n">
-        <v>311</v>
-      </c>
+        <v>13681</v>
+      </c>
+      <c r="G39" s="27" t="n"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>app</t>
@@ -2871,17 +2857,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-27 14:45:13</t>
+          <t>2026-10-27 15:27:47</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2891,13 +2877,15 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F40" s="27" t="n">
-        <v>4640</v>
-      </c>
-      <c r="G40" s="27" t="n"/>
+        <v>1401</v>
+      </c>
+      <c r="G40" s="27" t="n">
+        <v>311</v>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>app</t>
@@ -2907,7 +2895,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:39</t>
+          <t>2026-10-27 14:45:13</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2927,11 +2915,11 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F41" s="27" t="n">
-        <v>307</v>
+        <v>4640</v>
       </c>
       <c r="G41" s="27" t="n"/>
       <c r="H41" t="inlineStr">
@@ -2943,7 +2931,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-27 14:44:05</t>
+          <t>2026-10-27 14:44:39</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2963,11 +2951,11 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="F42" s="27" t="n">
-        <v>3787</v>
+        <v>307</v>
       </c>
       <c r="G42" s="27" t="n"/>
       <c r="H42" t="inlineStr">
@@ -2979,7 +2967,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-27 14:41:31</t>
+          <t>2026-10-27 14:44:05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2999,11 +2987,11 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F43" s="27" t="n">
-        <v>4947</v>
+        <v>3787</v>
       </c>
       <c r="G43" s="27" t="n"/>
       <c r="H43" t="inlineStr">
@@ -3015,17 +3003,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:15</t>
+          <t>2026-10-27 14:41:31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -3035,11 +3023,11 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F44" s="27" t="n">
-        <v>311</v>
+        <v>4947</v>
       </c>
       <c r="G44" s="27" t="n"/>
       <c r="H44" t="inlineStr">
@@ -3051,7 +3039,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-27 10:23:08</t>
+          <t>2026-10-27 10:23:15</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3071,15 +3059,13 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="F45" s="27" t="n">
-        <v>15809</v>
-      </c>
-      <c r="G45" s="27" t="n">
-        <v>1157</v>
-      </c>
+        <v>311</v>
+      </c>
+      <c r="G45" s="27" t="n"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>app</t>
@@ -3089,7 +3075,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-27 00:10:08</t>
+          <t>2026-10-27 10:23:08</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3104,16 +3090,30 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="n"/>
-      <c r="G46" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="F46" s="27" t="n">
+        <v>15809</v>
+      </c>
+      <c r="G46" s="27" t="n">
+        <v>1157</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-27 00:07:51</t>
+          <t>2026-10-27 00:10:08</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3128,40 +3128,26 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="F47" s="27" t="n">
-        <v>1157</v>
-      </c>
-      <c r="G47" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F47" s="27" t="n"/>
+      <c r="G47" s="27" t="n"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-27 00:02:49</t>
+          <t>2026-10-27 00:07:51</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3175,29 +3161,31 @@
         </is>
       </c>
       <c r="F48" s="27" t="n">
-        <v>8300</v>
-      </c>
-      <c r="G48" s="27" t="n"/>
+        <v>1157</v>
+      </c>
+      <c r="G48" s="27" t="n">
+        <v>911</v>
+      </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-26 14:42:55</t>
+          <t>2026-10-27 00:02:49</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3211,21 +3199,19 @@
         </is>
       </c>
       <c r="F49" s="27" t="n">
-        <v>911</v>
-      </c>
-      <c r="G49" s="27" t="n">
-        <v>351</v>
-      </c>
+        <v>8300</v>
+      </c>
+      <c r="G49" s="27" t="n"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:47</t>
+          <t>2026-10-26 14:42:55</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3249,9 +3235,11 @@
         </is>
       </c>
       <c r="F50" s="27" t="n">
+        <v>911</v>
+      </c>
+      <c r="G50" s="27" t="n">
         <v>351</v>
       </c>
-      <c r="G50" s="27" t="n"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>app</t>
@@ -3261,7 +3249,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-26 03:51:39</t>
+          <t>2026-10-26 03:51:47</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3281,15 +3269,13 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="F51" s="27" t="n">
-        <v>20274</v>
-      </c>
-      <c r="G51" s="27" t="n">
-        <v>3510</v>
-      </c>
+        <v>351</v>
+      </c>
+      <c r="G51" s="27" t="n"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>app</t>
@@ -3299,7 +3285,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-26 01:16:52</t>
+          <t>2026-10-26 03:51:39</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3323,10 +3309,10 @@
         </is>
       </c>
       <c r="F52" s="27" t="n">
+        <v>20274</v>
+      </c>
+      <c r="G52" s="27" t="n">
         <v>3510</v>
-      </c>
-      <c r="G52" s="27" t="n">
-        <v>351</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -3337,17 +3323,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-26 00:07:57</t>
+          <t>2026-10-26 01:16:52</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3361,29 +3347,31 @@
         </is>
       </c>
       <c r="F53" s="27" t="n">
-        <v>13001</v>
-      </c>
-      <c r="G53" s="27" t="n"/>
+        <v>3510</v>
+      </c>
+      <c r="G53" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-25 16:12:55</t>
+          <t>2026-10-26 00:07:57</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3397,19 +3385,19 @@
         </is>
       </c>
       <c r="F54" s="27" t="n">
-        <v>351</v>
+        <v>13001</v>
       </c>
       <c r="G54" s="27" t="n"/>
       <c r="H54" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-25 12:15:56</t>
+          <t>2026-10-25 16:12:55</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3424,16 +3412,28 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F55" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F55" s="27" t="n">
+        <v>351</v>
+      </c>
       <c r="G55" s="27" t="n"/>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-25 02:00:55</t>
+          <t>2026-10-25 12:15:56</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3448,40 +3448,26 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>2026-10-24</t>
-        </is>
-      </c>
-      <c r="F56" s="27" t="n">
-        <v>8060</v>
-      </c>
-      <c r="G56" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F56" s="27" t="n"/>
+      <c r="G56" s="27" t="n"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-25 00:11:33</t>
+          <t>2026-10-25 02:00:55</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3495,29 +3481,31 @@
         </is>
       </c>
       <c r="F57" s="27" t="n">
-        <v>7493</v>
-      </c>
-      <c r="G57" s="27" t="n"/>
+        <v>8060</v>
+      </c>
+      <c r="G57" s="27" t="n">
+        <v>122</v>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:21</t>
+          <t>2026-10-25 00:11:33</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3531,21 +3519,19 @@
         </is>
       </c>
       <c r="F58" s="27" t="n">
-        <v>122</v>
-      </c>
-      <c r="G58" s="27" t="n">
-        <v>121</v>
-      </c>
+        <v>7493</v>
+      </c>
+      <c r="G58" s="27" t="n"/>
       <c r="H58" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-24 16:46:10</t>
+          <t>2026-10-24 16:46:21</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3569,10 +3555,10 @@
         </is>
       </c>
       <c r="F59" s="27" t="n">
+        <v>122</v>
+      </c>
+      <c r="G59" s="27" t="n">
         <v>121</v>
-      </c>
-      <c r="G59" s="27" t="n">
-        <v>120</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -3583,7 +3569,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-24 08:35:48</t>
+          <t>2026-10-24 16:46:10</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3607,9 +3593,11 @@
         </is>
       </c>
       <c r="F60" s="27" t="n">
+        <v>121</v>
+      </c>
+      <c r="G60" s="27" t="n">
         <v>120</v>
       </c>
-      <c r="G60" s="27" t="n"/>
       <c r="H60" t="inlineStr">
         <is>
           <t>app</t>
@@ -3619,7 +3607,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-24 02:51:37</t>
+          <t>2026-10-24 08:35:48</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3639,15 +3627,13 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F61" s="27" t="n">
-        <v>8981</v>
-      </c>
-      <c r="G61" s="27" t="n">
-        <v>2680</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="G61" s="27" t="n"/>
       <c r="H61" t="inlineStr">
         <is>
           <t>app</t>
@@ -3657,7 +3643,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-24 01:14:58</t>
+          <t>2026-10-24 02:51:37</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3672,16 +3658,30 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F62" s="27" t="n"/>
-      <c r="G62" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F62" s="27" t="n">
+        <v>8981</v>
+      </c>
+      <c r="G62" s="27" t="n">
+        <v>2680</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-23 20:18:43</t>
+          <t>2026-10-24 01:14:58</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3696,40 +3696,26 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F63" s="27" t="n">
-        <v>2680</v>
-      </c>
-      <c r="G63" s="27" t="n">
-        <v>2650</v>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F63" s="27" t="n"/>
+      <c r="G63" s="27" t="n"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:58</t>
+          <t>2026-10-23 20:18:43</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3739,13 +3725,15 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F64" s="27" t="n">
-        <v>4933</v>
-      </c>
-      <c r="G64" s="27" t="n"/>
+        <v>2680</v>
+      </c>
+      <c r="G64" s="27" t="n">
+        <v>2650</v>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>app</t>
@@ -3755,7 +3743,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:45</t>
+          <t>2026-10-23 19:50:58</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3775,15 +3763,13 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F65" s="27" t="n">
-        <v>7567</v>
-      </c>
-      <c r="G65" s="27" t="n">
-        <v>0</v>
-      </c>
+        <v>4933</v>
+      </c>
+      <c r="G65" s="27" t="n"/>
       <c r="H65" t="inlineStr">
         <is>
           <t>app</t>
@@ -3793,7 +3779,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-23 19:50:27</t>
+          <t>2026-10-23 19:50:45</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3813,11 +3799,11 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F66" s="27" t="n">
-        <v>4189</v>
+        <v>7567</v>
       </c>
       <c r="G66" s="27" t="n">
         <v>0</v>
@@ -3831,7 +3817,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-23 19:49:41</t>
+          <t>2026-10-23 19:50:27</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3851,35 +3837,35 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F67" s="27" t="n">
-        <v>3685</v>
+        <v>4189</v>
       </c>
       <c r="G67" s="27" t="n">
         <v>0</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-23 18:21:22</t>
+          <t>2026-10-23 19:49:41</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3893,31 +3879,31 @@
         </is>
       </c>
       <c r="F68" s="27" t="n">
-        <v>2650</v>
+        <v>3685</v>
       </c>
       <c r="G68" s="27" t="n">
-        <v>831</v>
+        <v>0</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-23 15:07:26</t>
+          <t>2026-10-23 18:21:22</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3931,29 +3917,31 @@
         </is>
       </c>
       <c r="F69" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G69" s="27" t="n"/>
+        <v>2650</v>
+      </c>
+      <c r="G69" s="27" t="n">
+        <v>831</v>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-23 13:29:42</t>
+          <t>2026-10-23 15:07:26</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3967,21 +3955,19 @@
         </is>
       </c>
       <c r="F70" s="27" t="n">
-        <v>831</v>
-      </c>
-      <c r="G70" s="27" t="n">
-        <v>387</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G70" s="27" t="n"/>
       <c r="H70" t="inlineStr">
         <is>
-          <t>app</t>
+          <t>shortcut</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-23 09:09:43</t>
+          <t>2026-10-23 13:29:42</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3996,16 +3982,30 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F71" s="27" t="n"/>
-      <c r="G71" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="F71" s="27" t="n">
+        <v>831</v>
+      </c>
+      <c r="G71" s="27" t="n">
+        <v>387</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:26</t>
+          <t>2026-10-23 09:09:43</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4020,28 +4020,16 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="F72" s="27" t="n">
-        <v>387</v>
-      </c>
+          <t>synckey</t>
+        </is>
+      </c>
+      <c r="F72" s="27" t="n"/>
       <c r="G72" s="27" t="n"/>
-      <c r="H72" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-23 08:06:10</t>
+          <t>2026-10-23 08:06:26</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4061,15 +4049,13 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="F73" s="27" t="n">
-        <v>9720</v>
-      </c>
-      <c r="G73" s="27" t="n">
-        <v>1100</v>
-      </c>
+        <v>387</v>
+      </c>
+      <c r="G73" s="27" t="n"/>
       <c r="H73" t="inlineStr">
         <is>
           <t>app</t>
@@ -4079,17 +4065,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-23 01:18:21</t>
+          <t>2026-10-23 08:06:10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4103,9 +4089,11 @@
         </is>
       </c>
       <c r="F74" s="27" t="n">
-        <v>9097</v>
-      </c>
-      <c r="G74" s="27" t="n"/>
+        <v>9720</v>
+      </c>
+      <c r="G74" s="27" t="n">
+        <v>1100</v>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>app</t>
@@ -4115,31 +4103,43 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-22 17:45:58</t>
+          <t>2026-10-23 01:18:21</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F75" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F75" s="27" t="n">
+        <v>9097</v>
+      </c>
       <c r="G75" s="27" t="n"/>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-22 17:37:14</t>
+          <t>2026-10-22 17:45:58</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F76" s="27" t="n"/>
@@ -4163,53 +4163,41 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-22 15:53:11</t>
+          <t>2026-10-22 17:37:14</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F77" s="27" t="n">
-        <v>10808</v>
-      </c>
+          <t>requested</t>
+        </is>
+      </c>
+      <c r="F77" s="27" t="n"/>
       <c r="G77" s="27" t="n"/>
-      <c r="H77" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-22 15:25:40</t>
+          <t>2026-10-22 15:53:11</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4219,47 +4207,59 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F78" s="27" t="n">
-        <v>0</v>
+        <v>10808</v>
       </c>
       <c r="G78" s="27" t="n"/>
       <c r="H78" t="inlineStr">
         <is>
-          <t>shortcut</t>
+          <t>app</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-22 12:17:38</t>
+          <t>2026-10-22 15:25:40</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="F79" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="F79" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G79" s="27" t="n"/>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-22 11:21:02</t>
+          <t>2026-10-22 12:17:38</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="F80" s="27" t="n"/>
@@ -4283,22 +4283,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-22 11:06:21</t>
+          <t>2026-10-22 11:21:02</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>story</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F81" s="27" t="n"/>
@@ -4307,7 +4307,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:33</t>
+          <t>2026-10-22 11:06:21</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4322,28 +4322,16 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="F82" s="27" t="n">
-        <v>1100</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F82" s="27" t="n"/>
       <c r="G82" s="27" t="n"/>
-      <c r="H82" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-22 10:31:24</t>
+          <t>2026-10-22 10:31:33</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4363,15 +4351,13 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F83" s="27" t="n">
-        <v>18461</v>
-      </c>
-      <c r="G83" s="27" t="n">
-        <v>1985</v>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G83" s="27" t="n"/>
       <c r="H83" t="inlineStr">
         <is>
           <t>app</t>
@@ -4381,7 +4367,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:56</t>
+          <t>2026-10-22 10:31:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4396,16 +4382,30 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F84" s="27" t="n"/>
-      <c r="G84" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F84" s="27" t="n">
+        <v>18461</v>
+      </c>
+      <c r="G84" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-22 10:21:15</t>
+          <t>2026-10-22 10:21:56</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>unstory</t>
+          <t>story</t>
         </is>
       </c>
       <c r="F85" s="27" t="n"/>
@@ -4429,103 +4429,91 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-22 04:46:10</t>
+          <t>2026-10-22 10:21:15</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F86" s="27" t="n">
-        <v>4842</v>
-      </c>
+          <t>unstory</t>
+        </is>
+      </c>
+      <c r="F86" s="27" t="n"/>
       <c r="G86" s="27" t="n"/>
-      <c r="H86" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-22 03:50:41</t>
+          <t>2026-10-22 04:46:10</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>story</t>
-        </is>
-      </c>
-      <c r="F87" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F87" s="27" t="n">
+        <v>4842</v>
+      </c>
       <c r="G87" s="27" t="n"/>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-21 23:51:07</t>
+          <t>2026-10-22 03:50:41</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F88" s="27" t="n">
-        <v>0</v>
-      </c>
+          <t>story</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="n"/>
       <c r="G88" s="27" t="n"/>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>shortcut</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-21 23:49:15</t>
+          <t>2026-10-21 23:51:07</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4540,31 +4528,43 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F89" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F89" s="27" t="n">
+        <v>0</v>
+      </c>
       <c r="G89" s="27" t="n"/>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>shortcut</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-21 23:14:41</t>
+          <t>2026-10-21 23:49:15</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>minerva</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Minerva Perez</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F90" s="27" t="n"/>
@@ -4573,7 +4573,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-21 23:13:32</t>
+          <t>2026-10-21 23:14:41</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4588,28 +4588,16 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F91" s="27" t="n">
-        <v>12641</v>
-      </c>
+          <t>avatar</t>
+        </is>
+      </c>
+      <c r="F91" s="27" t="n"/>
       <c r="G91" s="27" t="n"/>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-21 23:11:16</t>
+          <t>2026-10-21 23:13:32</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4624,52 +4612,52 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F92" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F92" s="27" t="n">
+        <v>12641</v>
+      </c>
       <c r="G92" s="27" t="n"/>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-21 23:05:30</t>
+          <t>2026-10-21 23:11:16</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>armando</t>
+          <t>minerva</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Armando Alarcon</t>
+          <t>Minerva Perez</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F93" s="27" t="n">
-        <v>5345</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F93" s="27" t="n"/>
       <c r="G93" s="27" t="n"/>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:30</t>
+          <t>2026-10-21 23:05:30</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4684,16 +4672,28 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F94" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F94" s="27" t="n">
+        <v>5345</v>
+      </c>
       <c r="G94" s="27" t="n"/>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-10-21 23:04:04</t>
+          <t>2026-10-21 23:04:30</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F95" s="27" t="n"/>
@@ -4717,69 +4717,69 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-21 13:42:34</t>
+          <t>2026-10-21 23:04:04</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>armando</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Armando Alarcon</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F96" s="27" t="n">
-        <v>1985</v>
-      </c>
-      <c r="G96" s="27" t="n">
-        <v>100</v>
-      </c>
-      <c r="H96" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F96" s="27" t="n"/>
+      <c r="G96" s="27" t="n"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-21 13:12:27</t>
+          <t>2026-10-21 13:42:34</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>danielle</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Danielle Surini</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>avatar</t>
-        </is>
-      </c>
-      <c r="F97" s="27" t="n"/>
-      <c r="G97" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F97" s="27" t="n">
+        <v>1985</v>
+      </c>
+      <c r="G97" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-10-21 13:11:56</t>
+          <t>2026-10-21 13:12:27</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4794,7 +4794,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F98" s="27" t="n"/>
@@ -4803,43 +4803,31 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-10-21 12:36:32</t>
+          <t>2026-10-21 13:11:56</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>gonza</t>
+          <t>danielle</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Gonza Souza</t>
+          <t>Danielle Surini</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F99" s="27" t="n">
-        <v>10383</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F99" s="27" t="n"/>
       <c r="G99" s="27" t="n"/>
-      <c r="H99" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-10-21 12:28:14</t>
+          <t>2026-10-21 12:36:32</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4854,16 +4842,28 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F100" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F100" s="27" t="n">
+        <v>10383</v>
+      </c>
       <c r="G100" s="27" t="n"/>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-10-21 12:25:53</t>
+          <t>2026-10-21 12:28:14</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F101" s="27" t="n"/>
@@ -4887,43 +4887,31 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-21 11:03:58</t>
+          <t>2026-10-21 12:25:53</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>gonza</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Gonza Souza</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="F102" s="27" t="n">
-        <v>100</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F102" s="27" t="n"/>
       <c r="G102" s="27" t="n"/>
-      <c r="H102" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-21 11:01:42</t>
+          <t>2026-10-21 11:03:58</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4943,11 +4931,11 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F103" s="27" t="n">
-        <v>9060</v>
+        <v>100</v>
       </c>
       <c r="G103" s="27" t="n"/>
       <c r="H103" t="inlineStr">
@@ -4959,31 +4947,43 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-21 10:44:13</t>
+          <t>2026-10-21 11:01:42</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>luis</t>
+          <t>eron</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Luís Rodney</t>
+          <t>Eron Netto</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>synckey</t>
-        </is>
-      </c>
-      <c r="F104" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F104" s="27" t="n">
+        <v>9060</v>
+      </c>
       <c r="G104" s="27" t="n"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-10-21 10:43:02</t>
+          <t>2026-10-21 10:44:13</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F105" s="27" t="n"/>
@@ -5007,7 +5007,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-10-21 10:42:39</t>
+          <t>2026-10-21 10:43:02</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5022,7 +5022,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F106" s="27" t="n"/>
@@ -5031,43 +5031,31 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-10-21 04:34:33</t>
+          <t>2026-10-21 10:42:39</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>rogelio</t>
+          <t>luis</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Rogelio Garcia</t>
+          <t>Luís Rodney</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>steps</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="F107" s="27" t="n">
-        <v>6310</v>
-      </c>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F107" s="27" t="n"/>
       <c r="G107" s="27" t="n"/>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>app</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-10-21 03:05:30</t>
+          <t>2026-10-21 04:34:33</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5082,26 +5070,38 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>joined</t>
-        </is>
-      </c>
-      <c r="F108" s="27" t="n"/>
+          <t>steps</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F108" s="27" t="n">
+        <v>6310</v>
+      </c>
       <c r="G108" s="27" t="n"/>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-10-20 21:27:27</t>
+          <t>2026-10-21 03:05:30</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>helbert</t>
+          <t>rogelio</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Helbert Contreras</t>
+          <t>Rogelio Garcia</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -5115,7 +5115,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:09</t>
+          <t>2026-10-20 21:27:27</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5130,7 +5130,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F110" s="27" t="n"/>
@@ -5139,7 +5139,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-10-20 21:24:07</t>
+          <t>2026-10-20 21:24:09</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F111" s="27" t="n"/>
@@ -5163,7 +5163,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:48</t>
+          <t>2026-10-20 21:24:07</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>reset</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F112" s="27" t="n"/>
@@ -5187,7 +5187,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-10-20 21:23:44</t>
+          <t>2026-10-20 21:23:48</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5202,7 +5202,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>synckey</t>
+          <t>reset</t>
         </is>
       </c>
       <c r="F113" s="27" t="n"/>
@@ -5211,7 +5211,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-10-20 21:20:08</t>
+          <t>2026-10-20 21:23:44</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>synckey</t>
         </is>
       </c>
       <c r="F114" s="27" t="n"/>
@@ -5235,22 +5235,22 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-10-20 20:48:02</t>
+          <t>2026-10-20 21:20:08</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>eron</t>
+          <t>helbert</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Eron Netto</t>
+          <t>Helbert Contreras</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>joined</t>
         </is>
       </c>
       <c r="F115" s="27" t="n"/>
@@ -5259,7 +5259,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:34</t>
+          <t>2026-10-20 20:48:02</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5283,7 +5283,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-10-20 20:41:28</t>
+          <t>2026-10-20 20:41:34</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F117" s="27" t="n"/>
@@ -5307,7 +5307,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-10-20 20:27:02</t>
+          <t>2026-10-20 20:41:28</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F118" s="27" t="n"/>
@@ -5331,7 +5331,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-10-20 20:22:11</t>
+          <t>2026-10-20 20:27:02</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>denied</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F119" s="27" t="n"/>
@@ -5355,7 +5355,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-10-20 20:20:27</t>
+          <t>2026-10-20 20:22:11</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>requested</t>
+          <t>denied</t>
         </is>
       </c>
       <c r="F120" s="27" t="n"/>
@@ -5379,7 +5379,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-10-20 19:58:34</t>
+          <t>2026-10-20 20:20:27</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5403,7 +5403,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:19</t>
+          <t>2026-10-20 19:58:34</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>avatar</t>
+          <t>requested</t>
         </is>
       </c>
       <c r="F122" s="27" t="n"/>
@@ -5427,7 +5427,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-10-20 19:11:09</t>
+          <t>2026-10-20 19:11:19</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5442,11 +5442,35 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>joined</t>
+          <t>avatar</t>
         </is>
       </c>
       <c r="F123" s="27" t="n"/>
       <c r="G123" s="27" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:11:09</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>eron</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Eron Netto</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>joined</t>
+        </is>
+      </c>
+      <c r="F124" s="27" t="n"/>
+      <c r="G124" s="27" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>